<commit_message>
Update Excel files after daily scrape - 2026-09-13 07:06:28 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -79,7 +73,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,59 +496,59 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1316550</t>
+          <t>1339099</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1316550</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339099</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACE Program | Voice Spanish Translator</t>
+          <t>Architectural Design Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Sahibzada Ajit Singh Nagar, Punjab, India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>22 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services Ltd.</t>
+          <t>CGC JHANJERI MOHALI</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1338466</t>
+          <t>1339088</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338466</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339088</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Machine Learning Intern</t>
+          <t>Web development intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -570,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -587,22 +580,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338465</t>
+          <t>1339085</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338465</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339085</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Intern</t>
+          <t>Data Analyst Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sahibzada Ajit Singh Nagar, Punjab, India</t>
+          <t>Mullana, Haryana 133203, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -622,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CGC JHANJERI MOHALI</t>
+          <t>MM(DU) Mullana</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338464</t>
+          <t>1338978</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338464</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338978</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Electrical Engineering Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sahibzada Ajit Singh Nagar, Punjab, India</t>
+          <t>Mullana, Haryana 133203, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -664,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CGC JHANJERI MOHALI</t>
+          <t>MM(DU) Mullana</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1338115</t>
+          <t>1338289</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338115</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338289</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[Remote] Software Application Support and Development</t>
+          <t>Member Relations Manager</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No location available</t>
+          <t>Revora, Goa 403513, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -696,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>95 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>dJava Factory Sdn Bhd</t>
+          <t>Indulge Global</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1337434</t>
+          <t>1338079</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337434</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338079</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Customer Success Executive</t>
+          <t>Growth and Marketing Intern</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Córdoba, Argentina</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -738,59 +731,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>75 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Teleprom Argentina S.A</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1334167</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334167</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Cybersecurity Research Intern</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>M.A.H.E.</t>
+          <t>BeNinja Solutions</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-14 07:18:27 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="67" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339099</t>
+          <t>1339149</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339099</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339149</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Architectural Design Intern</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sahibzada Ajit Singh Nagar, Punjab, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CGC JHANJERI MOHALI</t>
+          <t>Aya Ehab Designs</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339088</t>
+          <t>1339127</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339088</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339127</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Web development intern</t>
+          <t>Social Media Specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sahibzada Ajit Singh Nagar, Punjab, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CGC JHANJERI MOHALI</t>
+          <t>BayanTech</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339085</t>
+          <t>1338812</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339085</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338812</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Data Analyst Intern</t>
+          <t>Data Analytics &amp; Planning Systems Trainee</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mullana, Haryana 133203, India</t>
+          <t>Breda, Hollandia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>178 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MM(DU) Mullana</t>
+          <t>Perfetti van Melle</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338978</t>
+          <t>1338586</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338978</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338586</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Electrical Engineering Intern</t>
+          <t>Social media specialist</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mullana, Haryana 133203, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MM(DU) Mullana</t>
+          <t>kremastos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1338289</t>
+          <t>1337983</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338289</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337983</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Member Relations Manager</t>
+          <t>[Partly Remote] Controlling Analyst HP 2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Revora, Goa 403513, India</t>
+          <t>Santiago, Región Metropolitana, Chile</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>42 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>Partly Remote</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Indulge Global</t>
+          <t>Boehringer Ingelheim in Chile</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1338079</t>
+          <t>1337958</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338079</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337958</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Growth and Marketing Intern</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>Altındere, 20050 Denizli Merkezefendi/Denizli, Türkiye</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,17 +731,605 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>53 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Özstar Kuruyemiş Makina Sanayi ve Ticaret Limited Şirketi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1336259</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336259</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Accounts Payable Clerk</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>47 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PSA Panama International Terminal, S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1334741</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334741</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Electrical Engineer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>64 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ETM MÜHENDİSLİK SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1334191</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334191</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Biotechnology Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>1 applicant</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>M.A.H.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1334159</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334159</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Computational Biomechanics Intern</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>BeNinja Solutions</t>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>M.A.H.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1333788</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1333788</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>88 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>GRATECH MAKİNA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1333592</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1333592</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>81 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>HORZUM DOKUMA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1332687</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332687</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Interpreter</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>26 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>KRAFT KİMYA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1332455</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332455</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Digital Marketer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>87 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ÇIRALI TEKSTİL İNŞAAT MÜHENDİSLİK VE MİMARLIK LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1332442</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332442</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sales Representative</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Honaz, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>37 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PAMUKKALE KURUYEMİŞ MAKİNALARI SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1331435</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331435</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SALES MANAGER</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Kumkısık, 20060 Denizli Merkezefendi/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>75 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>BEMOS OTOMASYON</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1329929</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1329929</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MARKETING &amp; SALES</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>58 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>DOĞAN İNŞ.MLZM.HAFR.NAK.İŞ MAK.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1327106</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1327106</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sales Assistant (Spanish)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>60 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Sera Moda</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1326081</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1326081</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>130 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ASM Crane</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1325856</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325856</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SALES ASSISTANT</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>91 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MULBERRY HOME</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-15 06:59:29 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="57" customWidth="1" min="4" max="4"/>
+    <col width="73" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="67" customWidth="1" min="8" max="8"/>
+    <col width="87" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339149</t>
+          <t>1339195</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339149</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339195</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Accelerate Romania - International Fundraising &amp; Friend-Raising Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Cluj-Napoca, Romania</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Aya Ehab Designs</t>
+          <t>Dog Assist</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339127</t>
+          <t>1339073</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339127</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339073</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Social Media Specialist</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Tanta, Tanta Qism 2, Tanta, Gharbia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BayanTech</t>
+          <t>PTCenter for physical therapy</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338812</t>
+          <t>1339072</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338812</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339072</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Planning Systems Trainee</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Breda, Hollandia</t>
+          <t>Tanta, Tanta Qism 2, Tanta, Gharbia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>178 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Perfetti van Melle</t>
+          <t>Otantik kumpir</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338586</t>
+          <t>1339071</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338586</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339071</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Social media specialist</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Tanta, Tanta Qism 2, Tanta, Gharbia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>kremastos</t>
+          <t>ITC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1337983</t>
+          <t>1338683</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337983</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338683</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[Partly Remote] Controlling Analyst HP 2026</t>
+          <t>Video Editor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Santiago, Región Metropolitana, Chile</t>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>42 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Partly Remote</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Boehringer Ingelheim in Chile</t>
+          <t>Eureka pharmaceuticals</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1337958</t>
+          <t>1338679</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337958</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338679</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>marketing specialist</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Altındere, 20050 Denizli Merkezefendi/Denizli, Türkiye</t>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,39 +731,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>53 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Özstar Kuruyemiş Makina Sanayi ve Ticaret Limited Şirketi</t>
+          <t>Eureka pharmaceuticals</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1336259</t>
+          <t>1338678</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336259</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338678</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Accounts Payable Clerk</t>
+          <t>Business Development Specialist</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,39 +773,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>47 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PSA Panama International Terminal, S.A.</t>
+          <t>Eureka pharmaceuticals</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1334741</t>
+          <t>1338627</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334741</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338627</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Electrical Engineer</t>
+          <t>Sales Represantative</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,39 +815,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>64 applicants</t>
+          <t>78 applicants</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ETM MÜHENDİSLİK SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>Enorm Teknoloji ve Yazılım Anonim Şirketi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1334191</t>
+          <t>1338163</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334191</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338163</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Biotechnology Intern</t>
+          <t>Business Developer</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Manipal, Karnataka, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,39 +857,39 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>M.A.H.E.</t>
+          <t>Orchida Soft</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1334159</t>
+          <t>1337244</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334159</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337244</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Computational Biomechanics Intern</t>
+          <t>Export Specialist in Istanbul</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Manipal, Karnataka, India</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,39 +899,39 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>36 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>M.A.H.E.</t>
+          <t>Akpa Aluminium</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1333788</t>
+          <t>1337083</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1333788</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337083</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>Digital Content and Marketing</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>88 applicants</t>
+          <t>215 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>GRATECH MAKİNA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>Capital Care Homes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1333592</t>
+          <t>1336355</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1333592</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336355</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>Regional Sales Representative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>81 applicants</t>
+          <t>55 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -993,29 +993,29 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HORZUM DOKUMA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>YILMAZ MAKİNE SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1332687</t>
+          <t>1332990</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332687</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332990</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Interpreter</t>
+          <t>Sales and Produciton Planning</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pamukkale, 20190 Pamukkale/Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1025,39 +1025,39 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>26 applicants</t>
+          <t>97 applicants</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>KRAFT KİMYA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>METAL MARKET DIŞ TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1332455</t>
+          <t>1332980</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332455</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332980</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Digital Marketer</t>
+          <t>Sales and Produciton Planning</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1067,39 +1067,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>87 applicants</t>
+          <t>105 applicants</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ÇIRALI TEKSTİL İNŞAAT MÜHENDİSLİK VE MİMARLIK LİMİTED ŞİRKETİ</t>
+          <t>METAL MARKET DIŞ TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1332442</t>
+          <t>1332703</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332442</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332703</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sales Representative</t>
+          <t>Sales Represantive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Honaz, Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>37 applicants</t>
+          <t>132 applicants</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1119,29 +1119,29 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>PAMUKKALE KURUYEMİŞ MAKİNALARI SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>KLT ENERJİ MÜHENDİSLİK</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1331435</t>
+          <t>1332481</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331435</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332481</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SALES MANAGER</t>
+          <t>Market Researcher</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kumkısık, 20060 Denizli Merkezefendi/Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>75 applicants</t>
+          <t>140 applicants</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1161,29 +1161,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BEMOS OTOMASYON</t>
+          <t>ÖZÇELİK MAKİNA SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1329929</t>
+          <t>1332032</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329929</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332032</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARKETING &amp; SALES</t>
+          <t>Sales Representative</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>58 applicants</t>
+          <t>141 applicants</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1203,29 +1203,29 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>DOĞAN İNŞ.MLZM.HAFR.NAK.İŞ MAK.SAN.VE TİC.LTD.ŞTİ.</t>
+          <t>Boğaziçi İhtisas Fuarcılık Limited Şirketi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1327106</t>
+          <t>1331747</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327106</t>
+          <t>https://aiesec.org/opportunity/global-talent/1331747</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sales Assistant (Spanish)</t>
+          <t>Sales Representative</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+          <t>Istanbul, İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1235,39 +1235,39 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>60 applicants</t>
+          <t>86 applicants</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Sera Moda</t>
+          <t>Apilex</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1326081</t>
+          <t>1323006</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1326081</t>
+          <t>https://aiesec.org/opportunity/global-talent/1323006</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing</t>
+          <t>OPERATIONS MANAGER</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+          <t>Kaklık, 20240 Honaz/Denizli, Türkiye</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>130 applicants</t>
+          <t>91 applicants</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1287,49 +1287,259 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ASM Crane</t>
+          <t>HEMMER MERMER MADENCİLİK İNŞAAT NAKLİYAT TURİZM İTHALAT İHRACAT SAN. VE TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1325856</t>
+          <t>1321833</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325856</t>
+          <t>https://aiesec.org/opportunity/global-talent/1321833</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SALES ASSISTANT</t>
+          <t>Digital Marketing</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>Gaziantep, Türkiye</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>142 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MACRO SIGN REKLAM İÇ VE DIŞ TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1321796</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1321796</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MARKET RESARCH &amp; MARKETİNG | ŞAHİNLER MARBLE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>Denizli, Kumkısık, Denizli, Türkiye</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>91 applicants</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>100 applicants</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>6 - 18 Months</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>MULBERRY HOME</t>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ŞAHİNLER MARBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1313381</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1313381</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sales Attendant</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Denizli, Kumkısık, Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>58 applicants</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>VAROL TEKSTİL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1307772</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1307772</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SALES and MARKETING - ZİMEK MAKİNE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Kocabaş, 20330 Honaz/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>144 applicants</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ZİMEK MAKİNA MERMER SAN. ve TİC. LTD ŞTİ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1303853</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1303853</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MARKETING &amp; SALES / ABC TEKSTİL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pınarkent, 20180 Pamukkale/Denizli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>146 applicants</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ABC TEKSTİL SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1288548</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1288548</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Market Researcher/Sales Assistant on Ergün Özen Machine</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Honaz, Türkiye</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>184 applicants</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ERGÜN ÖZEN MACHINA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-17 06:59:59 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="102" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339221</t>
+          <t>1339202</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339221</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339202</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Talent Management Intern</t>
+          <t>Sales Engineering</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panama City, Panamá Province, Panama</t>
+          <t>Gebze, Kocaeli, Türkiye</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+          <t>Mersen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339215</t>
+          <t>1339156</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339215</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339156</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>E-Commerce Senior Staff</t>
+          <t>HR Admin</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panama City, Panamá Province, Panama</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+          <t>Beta Trading Company</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339210</t>
+          <t>1339155</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339210</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339155</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sales Intern (German Market)</t>
+          <t>Business Development Officer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>HQ Solutions</t>
+          <t>Beta Trading Company</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1335628</t>
+          <t>1339016</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335628</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339016</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Marketer</t>
+          <t>Sales Responsible</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rades, Tunisia</t>
+          <t>Konya, Türkiye</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>32 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>AmazingPandph Digital Media Management</t>
+          <t>SRT Dişli Sanayi Anonim Şirketi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1327970</t>
+          <t>1338080</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327970</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338080</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Business Development Intern</t>
+          <t>Accelerate Romania | Italian-Speaking Purchasing &amp; Negotiation Specialist (EU Citizenship Required)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Malabe, Sri Lanka</t>
+          <t>Constanța, Romania</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,17 +689,269 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>49 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Veo Wordwide Services - Iași</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1337625</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337625</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Physiotherapy Intern</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Multan, Pakistan</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Barki Complex</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1337622</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337622</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Social Media Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Multan, Pakistan</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Barki Complex</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1331538</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331538</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Athens, Greece</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>286 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>3 - 6 Months</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Ribelz Integrated Pvt Ltd</t>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Dot by Dot</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1329177</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1329177</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[Impact Porto Alegre] - Social Media Intern – Intercultural Engagement Program</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Porto Alegre, RS, Brazil</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>115 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ESCOLA GIORDANO BRUNO LTDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1327760</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1327760</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fashion Consultant</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MPF clothing collection PVT LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1316755</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316755</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Kartepe, Kocaeli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>68 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Atom Mek</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-18 06:54:53 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,17 +445,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="102" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="103" customWidth="1" min="3" max="3"/>
+    <col width="79" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,32 +503,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339202</t>
+          <t>1339283</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339202</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339283</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sales Engineering</t>
+          <t>[EXP] Global customs services and surcharges specialist</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gebze, Kocaeli, Türkiye</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>9 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,113 +538,113 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mersen</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339156</t>
+          <t>1339288</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339156</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339288</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HR Admin</t>
+          <t>[CC] Change &amp; Transformation - Engagement Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Friedrich-Wilhelm-Straße 18, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>15 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Beta Trading Company</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339155</t>
+          <t>1339286</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339155</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339286</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Business Development Officer</t>
+          <t>[EXP] Global Internal Communications Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>13 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Beta Trading Company</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339016</t>
+          <t>1339230</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339016</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339230</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sales Responsible</t>
+          <t>Junior Sales Development Representative</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Konya, Türkiye</t>
+          <t>Galați, Romania</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +654,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SRT Dişli Sanayi Anonim Şirketi</t>
+          <t>CREATING ADITUDE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1338080</t>
+          <t>1339189</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338080</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339189</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Italian-Speaking Purchasing &amp; Negotiation Specialist (EU Citizenship Required)</t>
+          <t>Sales Representative (Spanish)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Constanța, Romania</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +696,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Veo Wordwide Services - Iași</t>
+          <t>OPINNATE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1337625</t>
+          <t>1339188</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337625</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339188</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Physiotherapy Intern</t>
+          <t>Sales Representative (German)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Multan, Pakistan</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,39 +738,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Barki Complex</t>
+          <t>OPINNATE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1337622</t>
+          <t>1339182</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337622</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339182</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Social Media Marketing Intern</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Multan, Pakistan</t>
+          <t>Ankara, Türkiye</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,39 +780,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Barki Complex</t>
+          <t>AHED Plastik</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1331538</t>
+          <t>1339181</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331538</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339181</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Athens, Greece</t>
+          <t>Ankara, Türkiye</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,39 +822,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>286 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Dot by Dot</t>
+          <t>AHED Plastik</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1329177</t>
+          <t>1339180</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329177</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339180</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[Impact Porto Alegre] - Social Media Intern – Intercultural Engagement Program</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Porto Alegre, RS, Brazil</t>
+          <t>Ankara, Türkiye</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,39 +864,39 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>115 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ESCOLA GIORDANO BRUNO LTDA</t>
+          <t>AHED Plastik</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1327760</t>
+          <t>1339108</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327760</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339108</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fashion Consultant</t>
+          <t>Marketing Professional</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,39 +906,39 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>MPF clothing collection PVT LTD</t>
+          <t>Ray IC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1316755</t>
+          <t>1339090</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1316755</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339090</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Marketing Specialist</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kartepe, Kocaeli, Türkiye</t>
+          <t>Ankara, Türkiye</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,17 +948,353 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>AHED Plastik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1338306</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338306</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>People Team Analyst</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>62 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1338121</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338121</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Marketing/Graphic Design Intern</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Santiago do Cacém, Portugal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>29 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Destilaria Black Pig Alentejo Unip. Lda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1337857</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337857</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Intern</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Charneca de Caparica, Portugal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>116 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Indústria dos Óculos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1337271</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337271</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>68 applicants</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>HILTI Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1337220</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337220</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Accelerate Romania | Junio Business Administrator / General Manager ( Moldova Citizenship Required )</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Piatra Neamț, Romania</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>50 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>SC LAPOOL SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1336117</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336117</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>UI/UX Research Intern</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1334121</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334121</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Nutrition and Dietetics Intern</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1331867</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331867</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sales Representative</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Istanbul, İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>75 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>3 - 6 Months</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Atom Mek</t>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>OPINNATE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-20 07:16:15 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="82" customWidth="1" min="4" max="4"/>
+    <col width="59" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339266</t>
+          <t>1339306</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339266</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339306</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Social media marketing</t>
+          <t>Social Media Manager</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kafr El-Shaikh, Qism Kafr El-Shaikh, Kafr el-Sheikh, Gharbia Governorate, Egypt</t>
+          <t>Sousse, Tunisia</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ITShop</t>
+          <t>Progress Professional Center</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339262</t>
+          <t>1339295</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339262</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339295</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mechanical Engineer</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
+          <t>Sousse, Tunisia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,34 +568,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Ray IC</t>
+          <t>Progress Professional Center</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339260</t>
+          <t>1337083</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339260</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337083</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Architecture Engineer</t>
+          <t>Digital Content and Marketing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>244 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Ray IC</t>
+          <t>Capital Care Homes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339213</t>
+          <t>1330854</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339213</t>
+          <t>https://aiesec.org/opportunity/global-talent/1330854</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>e-commerce specialist</t>
+          <t>Digital Production and e-commerce and Digital Assistance</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Kafr El-Shaikh, Qism Kafr El-Shaikh, Kafr el-Sheikh, Gharbia Governorate, Egypt</t>
+          <t>Αθήνα, Ελλάδα</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>76 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ITShop</t>
+          <t>Nanodomi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339208</t>
+          <t>1329104</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339208</t>
+          <t>https://aiesec.org/opportunity/global-talent/1329104</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Data Science Intern</t>
+          <t>Sales Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Jalandhar, Punjab, India</t>
+          <t>Pannipitiya, Sri Lanka</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,101 +689,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>58 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Lovely Professional University</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1336054</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336054</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>C# Developer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Alexandria, Alexandria Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>22 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>DotNet</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1327300</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327300</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Language Specialist - French</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Colombo, Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>54 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Aitken Spence Travels (Pvt) Ltd</t>
+          <t>Frella International</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-21 07:22:55 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="59" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="59" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="39" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339306</t>
+          <t>1339358</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339306</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339358</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Social Media Manager</t>
+          <t>Graphics and Design</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sousse, Tunisia</t>
+          <t>Ad Doqi, Dokki, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Progress Professional Center</t>
+          <t>Novel Creative House</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339295</t>
+          <t>1339284</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339295</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339284</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Web Developer</t>
+          <t>Social media specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sousse, Tunisia</t>
+          <t>Ad Doqi, Dokki, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Progress Professional Center</t>
+          <t>Novel Creative House</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1337083</t>
+          <t>1339277</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337083</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339277</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Digital Content and Marketing</t>
+          <t>Graphic design</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>244 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Capital Care Homes</t>
+          <t>Bybagh</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1330854</t>
+          <t>1339276</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1330854</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339276</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Production and e-commerce and Digital Assistance</t>
+          <t>Graphic design</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Αθήνα, Ελλάδα</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>76 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Nanodomi</t>
+          <t>Bybagh</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1329104</t>
+          <t>1339161</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329104</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339161</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sales Intern</t>
+          <t>Graphic design</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Pannipitiya, Sri Lanka</t>
+          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,17 +689,311 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>58 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bybagh</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1339160</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339160</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Business Development Associate</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bybagh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1339146</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339146</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Business Development Associate</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Bybagh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1339143</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339143</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Account manager</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>6th of October City, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Mediacs Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1339142</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339142</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Graphic design</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>6th of October City, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Mediacs Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1339141</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339141</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Business Development &amp; Client Strategy Executive</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>6th of October City, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Mediacs Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1339060</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339060</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Graphic designer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Clicks Creative Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1336318</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336318</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Financial Supervisor/Assistant Manager for Treasury</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>119 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>6 - 18 Months</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Frella International</t>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Innodays Business Management Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-22 07:09:54 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="54" customWidth="1" min="3" max="3"/>
-    <col width="59" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339358</t>
+          <t>1339384</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339358</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339384</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Graphics and Design</t>
+          <t>Sales Executive – Food &amp; Beverage</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ad Doqi, Dokki, Giza Governorate, Egypt</t>
+          <t>Alexandria, Alexandria Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Novel Creative House</t>
+          <t>cupofreel</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339284</t>
+          <t>1336712</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339284</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336712</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Social media specialist</t>
+          <t>Cloud Software Engineer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ad Doqi, Dokki, Giza Governorate, Egypt</t>
+          <t>Kavala, Greece</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>34 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Novel Creative House</t>
+          <t>Vertitech</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339277</t>
+          <t>1336200</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339277</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336200</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Graphic design</t>
+          <t>Business Development Executive (Remote)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Islamabad, Pakistan</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>30 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,24 +615,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>Dunya Consultants</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339276</t>
+          <t>1336047</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339276</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336047</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Graphic design</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>18 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>NOYO For Cosmetics</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339161</t>
+          <t>1336043</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339161</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Graphic design</t>
+          <t>Digital Marketing &amp; Media Buying Specialist</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>16 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>NOYO For Cosmetics</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339160</t>
+          <t>1335526</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339160</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335526</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Business Development Associate</t>
+          <t>Hotel Management Intern</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +741,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339146</t>
+          <t>1334122</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339146</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334122</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Business Development Associate</t>
+          <t>Forensic Science Intern</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt 5th settelement</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,29 +783,29 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339143</t>
+          <t>1334118</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339143</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334118</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Account manager</t>
+          <t>Law Intern</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>12 applicants</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -825,29 +825,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Mediacs Studio</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1339142</t>
+          <t>1334117</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339142</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334117</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Graphic design</t>
+          <t>Pharmacy Intern</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Mediacs Studio</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1339141</t>
+          <t>1334116</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339141</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334116</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Business Development &amp; Client Strategy Executive</t>
+          <t>Auditing and Taxation Intern</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>9 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,29 +909,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Mediacs Studio</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1339060</t>
+          <t>1334115</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339060</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334115</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Graphic designer</t>
+          <t>Business Administration Intern</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>17 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Clicks Creative Agency</t>
+          <t>Geeta University</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1336318</t>
+          <t>1334114</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336318</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334114</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Financial Supervisor/Assistant Manager for Treasury</t>
+          <t>Computer Science Engineering Intern</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Naultha, Haryana 132145, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,17 +983,311 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>119 applicants</t>
+          <t>13 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Innodays Business Management Limited</t>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1334112</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334112</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Human Resource Management Intern</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1334106</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334106</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Data Science and Business Analytics Intern</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1334102</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334102</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Full Stack Web Development Intern</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>4 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1334094</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334094</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cyber Security Intern</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>19 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1334089</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334089</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Machine Learning Intern</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>13 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1334085</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334085</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Finance Intern</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Naultha, Haryana 132145, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Geeta University</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1325604</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325604</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>International Business &amp; Innovation Analyst</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>4520 Santa Maria da Feira, Portugal</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>167 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>M2K Consultoria</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-24 07:06:58 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,17 +445,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="121" customWidth="1" min="3" max="3"/>
+    <col width="79" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,64 +503,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339384</t>
+          <t>1339488</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339384</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339488</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sales Executive – Food &amp; Beverage</t>
+          <t>[CC] UPGRADE Global Coordinator Talent Acquisition and Project Management (Only AIESECers. Fully read before applying)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Alexandria, Alexandria Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>20 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>cupofreel</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1336712</t>
+          <t>1339524</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336712</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339524</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cloud Software Engineer</t>
+          <t>Accounting Specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kavala, Greece</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +570,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>34 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Vertitech</t>
+          <t>Nestle Panama</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1336200</t>
+          <t>1339521</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336200</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339521</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Business Development Executive (Remote)</t>
+          <t>Marketing internship</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Novi Sad, Serbia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +612,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>30 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +622,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Dunya Consultants</t>
+          <t>DataDrill</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1336047</t>
+          <t>1339482</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336047</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339482</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>International Recruiter for Physiotherapists</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Groningen, Nederland</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +654,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>18 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NOYO For Cosmetics</t>
+          <t>Physiomatch</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1336043</t>
+          <t>1339471</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339471</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Digital Marketing &amp; Media Buying Specialist</t>
+          <t>Admission Counsellor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Visakhapatnam, Andhra Pradesh, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +696,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>16 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NOYO For Cosmetics</t>
+          <t>With Ease Education India Private Limited</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1335526</t>
+          <t>1339462</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335526</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339462</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hotel Management Intern</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +738,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +748,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>Candy Clan Studios</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1334122</t>
+          <t>1339461</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334122</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339461</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Forensic Science Intern</t>
+          <t>Interior Designer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,7 +780,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,29 +790,29 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>Candy Clan Studios</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1334118</t>
+          <t>1339456</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334118</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339456</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Law Intern</t>
+          <t>UI/UX Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,7 +822,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -825,29 +832,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1334117</t>
+          <t>1339455</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334117</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339455</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pharmacy Intern</t>
+          <t>Pharmacy Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +864,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,29 +874,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1334116</t>
+          <t>1339454</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334116</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339454</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Auditing and Taxation Intern</t>
+          <t>Law Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,7 +906,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>9 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,29 +916,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1334115</t>
+          <t>1339453</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334115</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339453</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Business Administration Intern</t>
+          <t>International Accounting Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,7 +948,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>17 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +958,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1334114</t>
+          <t>1339452</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334114</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339452</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Computer Science Engineering Intern</t>
+          <t>Human Resource Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,7 +990,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -993,29 +1000,29 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1334112</t>
+          <t>1339451</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334112</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339451</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Human Resource Management Intern</t>
+          <t>Hotel Management Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1025,7 +1032,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1035,29 +1042,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1334106</t>
+          <t>1339448</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334106</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339448</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Data Science and Business Analytics Intern</t>
+          <t>Game Design Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1067,7 +1074,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1077,29 +1084,29 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1334102</t>
+          <t>1339446</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334102</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339446</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Full Stack Web Development Intern</t>
+          <t>Full Stack Development Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1109,7 +1116,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1119,29 +1126,29 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1334094</t>
+          <t>1339442</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334094</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339442</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cyber Security Intern</t>
+          <t>Forensic Science Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1151,7 +1158,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>19 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1161,29 +1168,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1334089</t>
+          <t>1339441</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334089</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339441</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Artificial Intelligence and Machine Learning Intern</t>
+          <t>Finance Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1193,7 +1200,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>13 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1203,29 +1210,29 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1334085</t>
+          <t>1339435</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334085</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339435</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Finance Intern</t>
+          <t>Economics Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Naultha, Haryana 132145, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1235,7 +1242,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1245,29 +1252,29 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Geeta University</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1325604</t>
+          <t>1339433</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325604</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339433</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>International Business &amp; Innovation Analyst</t>
+          <t>Data Science Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4520 Santa Maria da Feira, Portugal</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1277,7 +1284,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>167 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1287,7 +1294,847 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>M2K Consultoria</t>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1339414</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339414</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Web Developer Intern</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ambala, Haryana, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MM(DU) Mullana</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1339394</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339394</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Computer Science Engineering Research Intern - 6 Weeks</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1339392</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339392</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Business Administration Research Intern - 6 Weeks</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1339281</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339281</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AI &amp; Computer Vision Developer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>6th of October City, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>icon studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1339259</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339259</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Electrical Engineer</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Ray IC</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1338889</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338889</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Prime Paper Products S.A.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1337761</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337761</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Export Manager Assistant</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>İzmir, Türkiye</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>122 applicants</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ACUNAL GIDA TARIM ÜRÜNLERİ MAKİNA İTHALAT İHRACAT SANAYİ VE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1336112</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336112</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Business Administration Research Intern</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>4 applicants</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1336111</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336111</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Computer Science Engineering Research Intern</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1335631</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1335631</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>content creator</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Tunis, Tunisie</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>22 applicants</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>citywork Business Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1335630</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1335630</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>community manager</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Tunis, Tunisie</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>8 applicants</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>citywork Business Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1335629</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1335629</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Brand strategist</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Tunis, Tunisie</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>14 applicants</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>citywork Business Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1334993</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334993</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>EXPORT MANAGER ASSISTANT</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>İzmir, Türkiye</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>142 applicants</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ACUNAL GIDA TARIM ÜRÜNLERİ MAKİNA İTHALAT İHRACAT SANAYİ VE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1332983</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332983</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Operations Control Support</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>96 applicants</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Nestle Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1331926</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331926</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Production Engineer</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>İzmir, Türkiye</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>86 applicants</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Norm Fasteners</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1331906</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331906</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Quality Engineer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>İzmir, Türkiye</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>71 applicants</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Norm Fasteners</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1330174</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1330174</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Accelerate Romania | Sales Specialist</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Timișoara, Romania</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>57 applicants</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Hibyte</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1328376</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1328376</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Export Manager Asistant</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>İzmir, Türkiye</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>150 applicants</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>BLACK LIGHT ELEKTRONIK SANAYI VE TICARET A.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1325344</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325344</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Customer Service for finance &amp; accounting (German Speaker)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>45 applicants</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>WMP Mexico Advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1317005</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1317005</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Manisa, Yunusemre/Manisa, Türkiye</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>245 applicants</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TOYO MATBAA MÜREKKEPLERİ SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-26 07:01:37 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -79,7 +73,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="115" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339548</t>
+          <t>1339591</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339548</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339591</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SALES at ROYAL FIRE SYSTEMS</t>
+          <t>A Design Experience Through Japanese Architecture by　TERASU — Illuminating the Future of  International Students</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
+          <t>日本、兵庫県宝塚市</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -538,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ROYAL FIRE SYSTEMS</t>
+          <t>Terasu Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339498</t>
+          <t>1339582</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339498</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339582</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Internatıonal Operations Specialist</t>
+          <t>Data Privacy and HS&amp;E Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>İstanbul, Türkiye</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -570,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>9 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -580,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Esenyel&amp;Partners Lawyers/Consultants</t>
+          <t>HILTI Panama</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339371</t>
+          <t>1339563</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339371</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339563</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Order-to-Invoice Trainee [EU Only]</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sofia, Bulgaria</t>
+          <t>Sousse, Tunisie</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>dormakaba</t>
+          <t>Sast Education</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339052</t>
+          <t>1339340</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339052</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339340</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Budget Control Sales Planning Sr. Analyst</t>
+          <t>Artificial Intelligence Research Intern 6 weeks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,227 +647,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>34 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Samsung Electronics Latinoamerica SELA Panama</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1338354</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338354</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>[DGF] Inside Sales Intern l German Speaker (EU Only)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Mainz, Germany</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>58 applicants</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>DHL Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1337973</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337973</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Sales at GEMSA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>40 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>GEMSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1336958</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336958</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Özsayın Soğutma Sistemleri</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>23 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Özsayın Soğutma Sistemleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1336432</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336432</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[Impact Brazil] - Content Creator and Engagement Intern</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>São Miguel do Oeste, SC, 89900-000, Brasil</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>19 applicants</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>KNN Idiomas</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1336043</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Digital Marketing &amp; Media Buying Specialist</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>16 applicants</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>NOYO For Cosmetics</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-27 07:29:16 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="115" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339591</t>
+          <t>1339525</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339591</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339525</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A Design Experience Through Japanese Architecture by　TERASU — Illuminating the Future of  International Students</t>
+          <t>Lawyer/ Legal Traniee</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>日本、兵庫県宝塚市</t>
+          <t>İstanbul, Türkiye</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Terasu Co., Ltd.</t>
+          <t>Esenyel&amp;Partners Lawyers/Consultants</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339582</t>
+          <t>1339106</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339582</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339106</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Data Privacy and HS&amp;E Intern</t>
+          <t>MARKETING EXECUTIVE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Birmingham, UK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>179 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>HILTI Panama</t>
+          <t>CROWNSOFT LTD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339563</t>
+          <t>1338536</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339563</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338536</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Voice Chat Product Operation - Spender</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sousse, Tunisie</t>
+          <t>中国上海市黄浦区</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>28 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Sast Education</t>
+          <t>PopUp</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339340</t>
+          <t>1337083</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339340</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337083</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Artificial Intelligence Research Intern 6 weeks</t>
+          <t>Digital Content and Marketing</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,17 +647,59 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>269 applicants</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Capital Care Homes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1335648</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1335648</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rajpura, Punjab, India</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>0 applicants</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>K.R. Mangalam University</t>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-28 07:57:30 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="41" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="57" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339525</t>
+          <t>1339463</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339525</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339463</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lawyer/ Legal Traniee</t>
+          <t>Brand Designer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>İstanbul, Türkiye</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Esenyel&amp;Partners Lawyers/Consultants</t>
+          <t>Candy Clan Studios</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339106</t>
+          <t>1338883</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339106</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338883</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MARKETING EXECUTIVE</t>
+          <t>Field Sales Employee (Aussendienstmitarbeiter)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Birmingham, UK</t>
+          <t>Berlin, Germany</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>179 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CROWNSOFT LTD</t>
+          <t>DewiBack Handels GmbH</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338536</t>
+          <t>1338882</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338536</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338882</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Voice Chat Product Operation - Spender</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>中国上海市黄浦区</t>
+          <t>Berlin, Germany</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>28 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PopUp</t>
+          <t>DewiBack Handels GmbH</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1337083</t>
+          <t>1338708</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337083</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338708</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Content and Marketing</t>
+          <t>Sales Development Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Nugegoda, Sri Lanka</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>269 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Capital Care Homes</t>
+          <t>Web Lankan Global (Pvt) Ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1335648</t>
+          <t>1337435</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335648</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337435</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing Intern</t>
+          <t>Digital Marketing and Sales Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rajpura, Punjab, India</t>
+          <t>Dehiwala-Mount Lavinia, Sri Lanka</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,17 +689,143 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>16 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>QJ Design Studios (PVT) LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1334342</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334342</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Electrical Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>M.A.H.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1330365</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1330365</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Creative Styling &amp; Brand Experience Intern</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MPF clothing collection PVT LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1327067</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1327067</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Creative Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>15 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MPF clothing collection PVT LTD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-29 07:53:42 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339463</t>
+          <t>1339665</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339463</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339665</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Brand Designer</t>
+          <t>[Impact Brazil] - Research &amp; Development Engineering Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Pouso Alegre, MG, 37550-000, Brasil</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Candy Clan Studios</t>
+          <t>Prática</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1338883</t>
+          <t>1339603</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338883</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339603</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Field Sales Employee (Aussendienstmitarbeiter)</t>
+          <t>Sales Representative</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Berlin, Germany</t>
+          <t>İzmir, Türkiye</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DewiBack Handels GmbH</t>
+          <t>Medstein</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338882</t>
+          <t>1338431</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338882</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338431</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>Public Relations and Marketing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Berlin, Germany</t>
+          <t>Dehradun, Uttarakhand, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DewiBack Handels GmbH</t>
+          <t>Cyber College Educational Society</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338708</t>
+          <t>1337649</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338708</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337649</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sales Development Intern</t>
+          <t>Clinical Study Operations Trainee</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>Brussels, Belgium</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,185 +647,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>61 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Web Lankan Global (Pvt) Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1337435</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337435</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Digital Marketing and Sales Intern</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Dehiwala-Mount Lavinia, Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>16 applicants</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>QJ Design Studios (PVT) LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1334342</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334342</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Electrical Engineer Intern</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>M.A.H.E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1330365</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1330365</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Creative Styling &amp; Brand Experience Intern</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>4 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>MPF clothing collection PVT LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1327067</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327067</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Creative Marketing Intern</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>15 applicants</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>MPF clothing collection PVT LTD</t>
+          <t>UCB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-09-30 07:44:39 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="86" customWidth="1" min="3" max="3"/>
+    <col width="41" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339665</t>
+          <t>1339713</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339665</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339713</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[Impact Brazil] - Research &amp; Development Engineering Intern</t>
+          <t>Talent Acquisition Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Pouso Alegre, MG, 37550-000, Brasil</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Prática</t>
+          <t>HILTI Panama</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339603</t>
+          <t>1339712</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339603</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339712</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sales Representative</t>
+          <t>Import Export Specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>İzmir, Türkiye</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Medstein</t>
+          <t>NESTRADE S.A, PANAMA BRANCH</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338431</t>
+          <t>1339697</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338431</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339697</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Public Relations and Marketing</t>
+          <t>Pre-construction Technician (Architecture)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Dehradun, Uttarakhand, India</t>
+          <t>Lisboa, Portugal</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cyber College Educational Society</t>
+          <t>Grupo Casais</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1337649</t>
+          <t>1339693</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337649</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339693</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Clinical Study Operations Trainee</t>
+          <t>Sustainable Tourism &amp; Community Development Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,17 +647,353 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>61 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Onevaasa Wilderness Labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1339679</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339679</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Inclusion Project Coordinator [EU Only]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1070 Anderlecht, Belgium</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>6 - 18 Months</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>UCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1339645</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339645</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Power Electronics Internship involving Inverter Experimentation and PSIM Simulation</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>日本、兵庫県神戸市</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sohatsu Systems Laboratory Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1339232</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339232</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Accelerate Romania | Location Manager Responsible</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Piatra Neamț, Romania</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SC La Popas SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1339231</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339231</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Accelerate Romania | Junior Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Piatra Neamț, Romania</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SC La Popas SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1338303</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338303</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Data &amp; AI Product Analyst</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>64 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Telered Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1337192</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337192</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Marketing Manager</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Arvicon International</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1323558</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1323558</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Construction Project Manager (Civil Engineer)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Lissabon, Portugal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>76 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Grupo Casais</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1316834</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316834</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Information Technology (IT) Analyst</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>102 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Özsayın Soğutma</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-01 08:07:33 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="86" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="108" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339713</t>
+          <t>1339519</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339713</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339519</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Talent Acquisition Intern</t>
+          <t>Sales &amp; Social Media Specialist</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,34 +526,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>HILTI Panama</t>
+          <t>ILux automation</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339712</t>
+          <t>1339379</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339712</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339379</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Import Export Specialist</t>
+          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - Spanish Speaker</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NESTRADE S.A, PANAMA BRANCH</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339697</t>
+          <t>1339378</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339697</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339378</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pre-construction Technician (Architecture)</t>
+          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - Spanish Speaker</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lisboa, Portugal</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Grupo Casais</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339693</t>
+          <t>1339376</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339693</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339376</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sustainable Tourism &amp; Community Development Intern</t>
+          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - Spanish Speaker</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ranchi, Jharkhand, India</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -652,34 +652,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Onevaasa Wilderness Labs</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339679</t>
+          <t>1339330</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339679</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339330</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Inclusion Project Coordinator [EU Only]</t>
+          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - Italian Speaker</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1070 Anderlecht, Belgium</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>UCB</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339645</t>
+          <t>1339329</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339645</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339329</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Power Electronics Internship involving Inverter Experimentation and PSIM Simulation</t>
+          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - German Speaker</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>日本、兵庫県神戸市</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -736,34 +736,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Sohatsu Systems Laboratory Inc.</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339232</t>
+          <t>1339327</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339232</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339327</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Location Manager Responsible</t>
+          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - French Speaker</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Piatra Neamț, Romania</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -778,34 +778,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SC La Popas SRL</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339231</t>
+          <t>1339326</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339231</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339326</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Junior Marketing Specialist</t>
+          <t>Accelerate Romania | Senior B2B Collections Analyst | EU Citizenship - German Speaker</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Piatra Neamț, Romania</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -820,34 +820,34 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SC La Popas SRL</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1338303</t>
+          <t>1339324</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338303</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339324</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Data &amp; AI Product Analyst</t>
+          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - German Speaker</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>64 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Telered Panama</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1337192</t>
+          <t>1339323</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337192</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339323</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Marketing Manager</t>
+          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - Italian Speaker</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi, India</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,39 +899,39 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Arvicon International</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1323558</t>
+          <t>1339322</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1323558</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339322</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Construction Project Manager (Civil Engineer)</t>
+          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - German Speaker</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lissabon, Portugal</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>76 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Grupo Casais</t>
+          <t>Genpact Iasi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1316834</t>
+          <t>1339305</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1316834</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339305</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Information Technology (IT) Analyst</t>
+          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - Italian Speaker</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
+          <t>Iași, Romania</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,17 +983,143 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>102 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Genpact Iasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1337278</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337278</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Regional BD Executive Americas</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>115 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PSA Panama International Terminal, S.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1335516</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1335516</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[EU/Brazil] C++ Software Development Intern (Linux and Rust)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>72 Tübingen, Germany</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>199 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Özsayın Soğutma</t>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Intra2net AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1332407</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332407</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Content Creator</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Infinitum Network Solutions</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-02 07:55:13 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,13 +445,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="108" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="86" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -496,74 +503,74 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339519</t>
+          <t>1339807</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339519</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339807</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sales &amp; Social Media Specialist</t>
+          <t>[CC] Talent Management &amp; Onboarding Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ILux automation</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339379</t>
+          <t>1339806</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339379</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339806</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - Spanish Speaker</t>
+          <t>[EXP NL] Business Analyst Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>15 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,39 +580,39 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339378</t>
+          <t>1339782</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339378</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339782</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - Spanish Speaker</t>
+          <t>[EXP] Internship Global BPO - Business Analyst team (EU Preferred)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>13 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,39 +622,39 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339376</t>
+          <t>1339781</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339376</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339781</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - Spanish Speaker</t>
+          <t>[EXP] Internship Global BPO - Business Analyst team (For Pre-Identified Candidate)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>19 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +664,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339330</t>
+          <t>1339700</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339330</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339700</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - Italian Speaker</t>
+          <t>Web Design</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +696,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>23 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +706,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>Corenet Tech Ltd.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339329</t>
+          <t>1339121</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339329</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339121</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - German Speaker</t>
+          <t>Finance Intern Controller</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>Panama City, Panamá Province, Panama</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +738,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>57 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +748,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>HILTI Panama</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339327</t>
+          <t>1338540</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339327</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338540</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Senior Financial Reporting &amp; Corporate Accountant | EU Citizenship - French Speaker</t>
+          <t>MARKETING</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>Bursa, Türkiye</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,49 +780,49 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>Modef Fuarcılık Ticaret Limited Şirketi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339326</t>
+          <t>1338472</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339326</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338472</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Senior B2B Collections Analyst | EU Citizenship - German Speaker</t>
+          <t>[EXP] Intern - Customer Emission Reporting</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>77 applicants</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -825,29 +832,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1339324</t>
+          <t>1338355</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339324</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338355</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - German Speaker</t>
+          <t>Procurement Support</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +864,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>79 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,29 +874,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>Nestle Panama</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1339323</t>
+          <t>1338273</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339323</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338273</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Intermediate Vendor Payments Specialist | EU Citizenship - Italian Speaker</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,7 +906,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>63 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,39 +916,39 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>Michael Page International Panamá S.A.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1339322</t>
+          <t>1338206</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339322</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338206</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - German Speaker</t>
+          <t>[EXP NL] Global Duty Billing Data Analytics Expert</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>161 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +958,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1339305</t>
+          <t>1337534</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339305</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337534</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Junior Invoice Processing Specialist| EU Citizenship - Italian Speaker</t>
+          <t>Market Analysis and Strategy Formulation Aim to Launch  Hair Care Products in India</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Iași, Romania</t>
+          <t>日本、東京都東京</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,39 +990,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>64 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Genpact Iasi</t>
+          <t>Milbon Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1337278</t>
+          <t>1337434</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337278</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337434</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Regional BD Executive Americas</t>
+          <t>Customer Success Executive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Córdoba, Argentina</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1025,7 +1032,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>115 applicants</t>
+          <t>85 applicants</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1035,29 +1042,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PSA Panama International Terminal, S.A.</t>
+          <t>Teleprom Argentina S.A</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1335516</t>
+          <t>1331618</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335516</t>
+          <t>https://aiesec.org/opportunity/global-talent/1331618</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[EU/Brazil] C++ Software Development Intern (Linux and Rust)</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>72 Tübingen, Germany</t>
+          <t>Aronj, Uttar Pradesh, India</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1067,39 +1074,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>199 applicants</t>
+          <t>15 applicants</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Intra2net AG</t>
+          <t>FS University</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1332407</t>
+          <t>1327512</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332407</t>
+          <t>https://aiesec.org/opportunity/global-talent/1327512</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Content Creator</t>
+          <t>Research Intern | Biotech</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Aronj, Uttar Pradesh, India</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1109,17 +1116,143 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>FS University</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1327511</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1327511</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>IT Interns</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Aronj, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>15 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>FS University</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1316696</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316696</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Biotech Intern</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Aronj, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>12 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Infinitum Network Solutions</t>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>FS University</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1304736</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1304736</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Hotel Entertainer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Heraklion, Greece</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>263 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Remarc Internation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-04 07:49:15 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="81" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339878</t>
+          <t>1339275</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339878</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339275</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Trainee ExCom</t>
+          <t>Graphic design</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>New Cairo City, Cairo Governorate, Egypt fifth settelment</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Adium Panama</t>
+          <t>Bybagh</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339876</t>
+          <t>1336079</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339876</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336079</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HR Analyst - People Transformation Hub</t>
+          <t>Brand Partner</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Adium Panama</t>
+          <t>Rediffusion Brand Solutions Pvt Ltd</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339840</t>
+          <t>1336078</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339840</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336078</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sales Intern (German Market)</t>
+          <t>Design Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Levata by Logiscenter</t>
+          <t>Rediffusion Brand Solutions Pvt Ltd</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339371</t>
+          <t>1317568</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339371</t>
+          <t>https://aiesec.org/opportunity/global-talent/1317568</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Order-to-Invoice Trainee [EU Only]</t>
+          <t>Research Intern, Project base learning</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sofia, Bulgaria</t>
+          <t>Pune, Maharashtra, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10 applicants</t>
+          <t>40 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>dormakaba</t>
+          <t>PVG’s College of Engineering and Technology</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1325830</t>
+          <t>1293818</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325830</t>
+          <t>https://aiesec.org/opportunity/global-talent/1293818</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing Intern</t>
+          <t>Receptionist and Sales Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Makati City, Metro Manila, Philippines</t>
+          <t>Chalkidiki, Greece</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,59 +689,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>61 applicants</t>
+          <t>275 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Consistent Frozen Solutions Corporation</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1299853</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1299853</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>[Impact Porto Alegre] - Social Media Intern – Intercultural Engagement Program</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Porto Alegre, RS, Brasil</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>172 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ESCOLA GIORDANO BRUNO LTDA</t>
+          <t>Hotel Kriopigi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-05 08:03:25 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="41" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="43" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339275</t>
+          <t>1339870</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339275</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339870</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Graphic design</t>
+          <t>Project Specialist</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt fifth settelment</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>10 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Bybagh</t>
+          <t>NESTRADE S.A, PANAMA BRANCH</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1336079</t>
+          <t>1339756</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336079</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339756</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Brand Partner</t>
+          <t>Architectural Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>Dehradun, Uttarakhand, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rediffusion Brand Solutions Pvt Ltd</t>
+          <t>Archana Kapil Associates Private Limited</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1336078</t>
+          <t>1339755</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336078</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339755</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Design Intern</t>
+          <t>Business Development And Marketing Strategist</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Rediffusion Brand Solutions Pvt Ltd</t>
+          <t>DMG Technologies</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1317568</t>
+          <t>1339754</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1317568</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339754</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Research Intern, Project base learning</t>
+          <t>Full-Stack Software Developer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>40 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PVG’s College of Engineering and Technology</t>
+          <t>DMG Technologies</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1293818</t>
+          <t>1339753</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1293818</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339753</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Receptionist and Sales Intern</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Chalkidiki, Greece</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>275 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,7 +699,49 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Hotel Kriopigi</t>
+          <t>DMG Technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1339704</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339704</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Bussiness Developer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cairo, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Loc-Gate</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-06 08:30:53 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -443,12 +443,12 @@
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="43" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339870</t>
+          <t>1339980</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339870</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339980</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Project Specialist</t>
+          <t>Business Development &amp; Growth Marketing Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Saltillo, Coahuila, Mexico</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NESTRADE S.A, PANAMA BRANCH</t>
+          <t>Manover MX</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339756</t>
+          <t>1339978</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339756</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339978</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Architectural Intern</t>
+          <t>Industrial Projects &amp; Engineering Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Dehradun, Uttarakhand, India</t>
+          <t>Saltillo, Coahuila, Mexico</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,34 +568,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Archana Kapil Associates Private Limited</t>
+          <t>Manover MX</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339755</t>
+          <t>1339977</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339755</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339977</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Business Development And Marketing Strategist</t>
+          <t>Sourcing Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DMG Technologies</t>
+          <t>Adison Partners</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339754</t>
+          <t>1339881</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339754</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339881</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Full-Stack Software Developer</t>
+          <t>Marketer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DMG Technologies</t>
+          <t>Ateco</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339753</t>
+          <t>1335301</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339753</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335301</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Technical Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>22 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DMG Technologies</t>
+          <t>ZOHO Corporation</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339704</t>
+          <t>1331894</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339704</t>
+          <t>https://aiesec.org/opportunity/global-talent/1331894</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bussiness Developer</t>
+          <t>Sales Engineer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Kartepe, Kocaeli, Türkiye</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>100 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Loc-Gate</t>
+          <t>Atom Mek</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-07 08:08:51 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339980</t>
+          <t>1339925</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339980</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339925</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Growth Marketing Intern</t>
+          <t>Content &amp; Social Media Marketing Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Saltillo, Coahuila, Mexico</t>
+          <t>Unawatuna, Sri Lanka</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Manover MX</t>
+          <t>Angel Beach Club Unawatuna</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339978</t>
+          <t>1339917</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339978</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339917</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Industrial Projects &amp; Engineering Intern</t>
+          <t>UI/UX Designer Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Saltillo, Coahuila, Mexico</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Manover MX</t>
+          <t>VirtualCity Informatics Pvt. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339977</t>
+          <t>1339915</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339977</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339915</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sourcing Intern</t>
+          <t>UI/UX Designer Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Adison Partners</t>
+          <t>VirtualCity Informatics Pvt. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339881</t>
+          <t>1339893</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339881</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339893</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Marketer</t>
+          <t>Marketing and Research - Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Nugegoda, Sri Lanka</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Ateco</t>
+          <t>Xiteb (Pvt) Ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1335301</t>
+          <t>1339892</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335301</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339892</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Technical Intern</t>
+          <t>Intern Project Analyst</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Nugegoda, Sri Lanka</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>22 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ZOHO Corporation</t>
+          <t>Xiteb (Pvt) Ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1331894</t>
+          <t>1339885</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331894</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339885</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sales Engineer</t>
+          <t>Social media marketing</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Kartepe, Kocaeli, Türkiye</t>
+          <t>Amman, Jordan</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,17 +731,437 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>100 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Kalamantina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1339847</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339847</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ai Intern</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SKIPS University</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1339772</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339772</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Human Resource Intern</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rajpura, Punjab, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1338740</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338740</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Marketing Assistant Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nugegoda, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>3 - 6 Months</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Atom Mek</t>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Brand Corridor (Pvt) Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1338739</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338739</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trainee Accounting Intern</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nugegoda, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Brand Corridor (Pvt) Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1336041</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336041</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Administrative, Marketing &amp; E-Marketing (Fairs, Events &amp;  Customer Follow-up)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cairo, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>15 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NAGEH ENGINEERING CO.- LLC شركة ناجح الهندسية</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1336040</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336040</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Aviation Engineer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Cairo, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>20 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NAGEH ENGINEERING CO.- LLC شركة ناجح الهندسية</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1332408</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332408</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Content Writer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Infinitum Network Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1329526</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1329526</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[Impact Brazil] - Supplier Development Procurement Intern</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Joinville - Pirabeiraba, Joinville - SC, Brasil</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>122 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Nidec Global Appliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1325832</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325832</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Inventory Management Intern</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Makati City, Metro Manila, Philippines</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>75 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Consistent Frozen Solutions Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1325829</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325829</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Business Process Management Intern</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Makati City, Metro Manila, Philippines</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>69 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Consistent Frozen Solutions Corporation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-08 08:26:15 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,16 +445,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="86" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -496,22 +503,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339925</t>
+          <t>1340008</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339925</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340008</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Content &amp; Social Media Marketing Intern</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unawatuna, Sri Lanka</t>
+          <t>Abidjan, Côte d'Ivoire</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +528,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Angel Beach Club Unawatuna</t>
+          <t>AQUALIS INGENIEUR CONSEIL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339917</t>
+          <t>1339873</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339917</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339873</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UI/UX Designer Intern</t>
+          <t>Business Consultant</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +570,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>VirtualCity Informatics Pvt. Ltd.</t>
+          <t>Ergonx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339915</t>
+          <t>1339871</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339915</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339871</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UI/UX Designer Intern</t>
+          <t>Application Security (AppSec) Engineer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -615,29 +622,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>VirtualCity Informatics Pvt. Ltd.</t>
+          <t>Riva Talent</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339893</t>
+          <t>1339767</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339893</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339767</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Marketing and Research - Intern</t>
+          <t>Mechanical Engineering Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>Rajpura, Punjab, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -652,34 +659,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Xiteb (Pvt) Ltd</t>
+          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339892</t>
+          <t>1339766</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339892</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339766</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Intern Project Analyst</t>
+          <t>Civil Engineering Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>Rajpura, Punjab, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +696,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Xiteb (Pvt) Ltd</t>
+          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339885</t>
+          <t>1339710</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339885</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339710</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Social media marketing</t>
+          <t>Frontend developer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Amman, Jordan</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +738,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +748,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Kalamantina</t>
+          <t>Riva Talent</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339847</t>
+          <t>1339706</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339847</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339706</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ai Intern</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat, India</t>
+          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -783,29 +790,29 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SKIPS University</t>
+          <t>Riva Talent</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339772</t>
+          <t>1339486</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339772</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339486</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Human Resource Intern</t>
+          <t>IT (6 weeks!)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Rajpura, Punjab, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -825,29 +832,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
+          <t>home mart reality</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1338740</t>
+          <t>1339485</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338740</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339485</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Marketing Assistant Intern</t>
+          <t>Sales (6 weeks!)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -862,34 +869,34 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Brand Corridor (Pvt) Ltd</t>
+          <t>home mart reality</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1338739</t>
+          <t>1339481</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338739</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339481</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Trainee Accounting Intern</t>
+          <t>Digital marketing  (6 weeks!)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,34 +906,34 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Brand Corridor (Pvt) Ltd</t>
+          <t>home mart reality</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1336041</t>
+          <t>1339359</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336041</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339359</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Administrative, Marketing &amp; E-Marketing (Fairs, Events &amp;  Customer Follow-up)</t>
+          <t>Interior Designer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -941,7 +948,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -951,29 +958,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NAGEH ENGINEERING CO.- LLC شركة ناجح الهندسية</t>
+          <t>Ergonx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1336040</t>
+          <t>1338821</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336040</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338821</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Aviation Engineer</t>
+          <t>Clinical Site Associate Trainee [ EU Only]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>1070 Anderlecht, Belgium</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,39 +990,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>20 applicants</t>
+          <t>24 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NAGEH ENGINEERING CO.- LLC شركة ناجح الهندسية</t>
+          <t>UCB</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1332408</t>
+          <t>1337875</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332408</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337875</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Content Writer</t>
+          <t>Business Development</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Ankara, Türkiye</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1025,39 +1032,39 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>88 applicants</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Infinitum Network Solutions</t>
+          <t>Akın Global Medikal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1329526</t>
+          <t>1337808</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329526</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337808</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[Impact Brazil] - Supplier Development Procurement Intern</t>
+          <t>Sales &amp; Impact Trainee</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Joinville - Pirabeiraba, Joinville - SC, Brasil</t>
+          <t>Brussels, Belgium</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1067,39 +1074,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>122 applicants</t>
+          <t>129 applicants</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Nidec Global Appliance</t>
+          <t>Shayp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1325832</t>
+          <t>1337534</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325832</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337534</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inventory Management Intern</t>
+          <t>Market Analysis and Strategy Formulation Aim to Launch  Hair Care Products in India</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Makati City, Metro Manila, Philippines</t>
+          <t>日本、東京都東京</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1109,39 +1116,39 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>75 applicants</t>
+          <t>64 applicants</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Consistent Frozen Solutions Corporation</t>
+          <t>Milbon Co., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1325829</t>
+          <t>1336846</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325829</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336846</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Business Process Management Intern</t>
+          <t>Accelerate Romania - Process Engineering Intern – AEC Workflows</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Makati City, Metro Manila, Philippines</t>
+          <t>Satu Mare, Romania</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1151,17 +1158,227 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>69 applicants</t>
+          <t>34 applicants</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Parametric Design Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1334440</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334440</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Civil Engineering Intern</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>M.A.H.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1332411</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332411</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Infinitum Network Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1332409</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332409</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Youtube Manager</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Infinitum Network Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1331811</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331811</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>[EXP] Global Digital Marketing Intern – Content &amp; Social Media</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>312 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>DHL Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1304488</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1304488</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Client Consultant | Tourism Sector (German /Dutch speaker) ( Flexible RE dates )</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Athens, Greece</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>103 applicants</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>3 - 6 Months</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Consistent Frozen Solutions Corporation</t>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SpeakIT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-09 08:23:51 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -79,7 +73,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="86" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="57" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340008</t>
+          <t>1340098</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340008</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340098</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Controlling Analyst AH 2027</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Abidjan, Côte d'Ivoire</t>
+          <t>Santiago, Región Metropolitana, Chile</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>AQUALIS INGENIEUR CONSEIL</t>
+          <t>Boehringer Ingelheim in Chile</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1339873</t>
+          <t>1340096</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339873</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340096</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Business Consultant</t>
+          <t>MARKETING ANALYST 2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Santiago, Región Metropolitana, Chile</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -570,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Ergonx</t>
+          <t>Boehringer Ingelheim in Chile</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339871</t>
+          <t>1340094</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339871</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340094</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Application Security (AppSec) Engineer</t>
+          <t>Marketing Analyst 2027</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Santiago, Región Metropolitana, Chile</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Riva Talent</t>
+          <t>Boehringer Ingelheim in Chile</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339767</t>
+          <t>1340088</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339767</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340088</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Intern</t>
+          <t>Services Procurement &amp; Project Operations Analyst</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rajpura, Punjab, India</t>
+          <t>Santiago, Región Metropolitana, Chile</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
+          <t>Philips Chilena</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339766</t>
+          <t>1340061</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339766</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340061</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Civil Engineering Intern</t>
+          <t>Sales Engineer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rajpura, Punjab, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -696,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -706,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Swami Vivekanand Institute of Engineering &amp; Technology</t>
+          <t>Expert Smart</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339710</t>
+          <t>1340000</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339710</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340000</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Frontend developer</t>
+          <t>Business Coordinator</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -738,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -748,29 +741,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Riva Talent</t>
+          <t>Ma maisonnette</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339706</t>
+          <t>1339999</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339706</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339999</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
+          <t>Business Coordinator</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
+          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -780,7 +773,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -790,29 +783,29 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Riva Talent</t>
+          <t>Ma maisonnette</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339486</t>
+          <t>1339615</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339486</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339615</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>IT (6 weeks!)</t>
+          <t>Social media photographer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Alexandria, Alexandria Governorate, Egypt</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -822,7 +815,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -832,29 +825,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>home mart reality</t>
+          <t>TFH The Fit Hub</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1339485</t>
+          <t>1335631</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339485</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335631</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sales (6 weeks!)</t>
+          <t>content creator</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Tunis, Tunisie</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -864,7 +857,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>22 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -874,29 +867,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>home mart reality</t>
+          <t>citywork Business Center</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1339481</t>
+          <t>1335630</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339481</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335630</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Digital marketing  (6 weeks!)</t>
+          <t>community manager</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Tunis, Tunisie</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -906,7 +899,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>9 applicants</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -916,29 +909,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>home mart reality</t>
+          <t>citywork Business Center</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1339359</t>
+          <t>1334355</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339359</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334355</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Interior Designer</t>
+          <t>AI Intern</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Manipal, Karnataka, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -948,39 +941,39 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>21 applicants</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Ergonx</t>
+          <t>MAHE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1338821</t>
+          <t>1307772</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338821</t>
+          <t>https://aiesec.org/opportunity/global-talent/1307772</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Clinical Site Associate Trainee [ EU Only]</t>
+          <t>SALES and MARKETING - ZİMEK MAKİNE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1070 Anderlecht, Belgium</t>
+          <t>Kocabaş, 20330 Honaz/Denizli, Türkiye</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -990,7 +983,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>24 applicants</t>
+          <t>148 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1000,385 +993,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>UCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1337875</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337875</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Business Development</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Ankara, Türkiye</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>88 applicants</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Akın Global Medikal</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1337808</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337808</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Sales &amp; Impact Trainee</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Brussels, Belgium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>129 applicants</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Shayp</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1337534</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337534</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Market Analysis and Strategy Formulation Aim to Launch  Hair Care Products in India</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>日本、東京都東京</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>64 applicants</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Milbon Co., Ltd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1336846</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336846</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Accelerate Romania - Process Engineering Intern – AEC Workflows</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Satu Mare, Romania</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>34 applicants</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Parametric Design Solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1334440</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334440</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Civil Engineering Intern</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>0 applicants</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>M.A.H.E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1332411</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332411</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Director</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2 applicants</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Infinitum Network Solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1332409</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332409</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Youtube Manager</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Infinitum Network Solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1331811</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331811</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>[EXP] Global Digital Marketing Intern – Content &amp; Social Media</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Maastricht, Netherlands</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>312 applicants</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>DHL Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1304488</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1304488</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Client Consultant | Tourism Sector (German /Dutch speaker) ( Flexible RE dates )</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Athens, Greece</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>103 applicants</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>SpeakIT</t>
+          <t>ZİMEK MAKİNA MERMER SAN. ve TİC. LTD ŞTİ.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-10 08:11:38 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340098</t>
+          <t>1340059</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340098</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340059</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Controlling Analyst AH 2027</t>
+          <t>Film making</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Santiago, Región Metropolitana, Chile</t>
+          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Boehringer Ingelheim in Chile</t>
+          <t>Baynoire</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340096</t>
+          <t>1338341</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340096</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338341</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MARKETING ANALYST 2026</t>
+          <t>Growth and Marketing Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Santiago, Región Metropolitana, Chile</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,34 +568,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Boehringer Ingelheim in Chile</t>
+          <t>BeNinja Solutions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340094</t>
+          <t>1334352</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340094</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334352</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Marketing Analyst 2027</t>
+          <t>AI Research Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Santiago, Región Metropolitana, Chile</t>
+          <t>Manipal, Karnataka, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Boehringer Ingelheim in Chile</t>
+          <t>MAHE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340088</t>
+          <t>1334345</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340088</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334345</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Services Procurement &amp; Project Operations Analyst</t>
+          <t>AI Research Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Santiago, Región Metropolitana, Chile</t>
+          <t>Manipal, Karnataka, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Philips Chilena</t>
+          <t>MAHE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1340061</t>
+          <t>1334182</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340061</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334182</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sales Engineer</t>
+          <t>Robotics Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Manipal, Karnataka, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Expert Smart</t>
+          <t>M.A.H.E.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1340000</t>
+          <t>1332403</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340000</t>
+          <t>https://aiesec.org/opportunity/global-talent/1332403</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Business Coordinator</t>
+          <t>Actor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,259 +741,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Ma maisonnette</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1339999</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339999</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Business Coordinator</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Ma maisonnette</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1339615</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339615</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Social media photographer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Alexandria, Alexandria Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>TFH The Fit Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1335631</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335631</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>content creator</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Tunis, Tunisie</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>22 applicants</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>citywork Business Center</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1335630</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335630</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>community manager</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Tunis, Tunisie</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>9 applicants</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>citywork Business Center</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1334355</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334355</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>AI Intern</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>21 applicants</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1307772</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1307772</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>SALES and MARKETING - ZİMEK MAKİNE</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Kocabaş, 20330 Honaz/Denizli, Türkiye</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>148 applicants</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>ZİMEK MAKİNA MERMER SAN. ve TİC. LTD ŞTİ.</t>
+          <t>Infinitum Network Solutions</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-11 08:15:43 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,16 +438,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340059</t>
+          <t>1339420</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340059</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339420</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Film making</t>
+          <t>studio trainer (classes trainer)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>El Sheikh Zayed City, Giza Governorate, Egypt</t>
+          <t>Alexandria, Alexandria Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Baynoire</t>
+          <t>TFH The Fit Hub</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1338341</t>
+          <t>1339296</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338341</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339296</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Growth and Marketing Intern</t>
+          <t>Receptionist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>Thanh Thủy, Phú Thọ, Việt Nam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BeNinja Solutions</t>
+          <t>LYNN TIMES HOTELS &amp; RESORTS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1334352</t>
+          <t>1337863</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334352</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337863</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AI Research Intern</t>
+          <t>Social Media Specialist</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Manipal, Karnataka, India</t>
+          <t>中国广东省深圳市龙岗区</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,143 +605,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>98 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1334345</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334345</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>AI Research Intern</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>4 applicants</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1334182</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334182</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Robotics Intern</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>6 applicants</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>M.A.H.E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1332403</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1332403</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Infinitum Network Solutions</t>
+          <t>Keychron</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-12 08:23:45 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,16 +438,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339420</t>
+          <t>1339308</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339420</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339308</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>studio trainer (classes trainer)</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Alexandria, Alexandria Governorate, Egypt</t>
+          <t>Thanh Thủy, Phú Thọ, Việt Nam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,91 +531,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TFH The Fit Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1339296</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339296</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Receptionist</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Thanh Thủy, Phú Thọ, Việt Nam</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>3 applicants</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>LYNN TIMES HOTELS &amp; RESORTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1337863</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337863</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Social Media Specialist</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>中国广东省深圳市龙岗区</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>98 applicants</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Keychron</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-13 08:46:32 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,17 +445,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="71" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,42 +503,546 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1339308</t>
+          <t>1338354</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339308</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338354</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>[DGF] Inside Sales Intern l German Speaker (EU Only)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thanh Thủy, Phú Thọ, Việt Nam</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+          <t>Mainz, Germany</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>70 applicants</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>DHL Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1338472</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338472</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[EXP] Intern - Customer Emission Reporting</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>117 applicants</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>DHL Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1340175</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340175</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Accelerate Romania - Junior Marketing &amp; Growth Specialist</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Baia Mare, Romania</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2 applicants</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>LYNN TIMES HOTELS &amp; RESORTS</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Coach Jurnal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1340039</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340039</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Junior Hardware Engineer (EPLAN) – Marine Automation (Preferably EU)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Delft, Nederland</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Smart-Ship B.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1338115</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338115</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[Remote] Software Application Support and Development</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No location available</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>126 applicants</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>dJava Factory Sdn Bhd</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1336624</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336624</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Business Development Executive</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Galle, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>17 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sanmark Solutions Pvt Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1336109</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336109</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data Science Research Intern</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>10 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1336107</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336107</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cyber Security Research Intern</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>18 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1336106</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336106</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Research Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>12 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1327760</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1327760</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fashion Consultant</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MPF clothing collection PVT LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1325297</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1325297</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>International Sales Representetive Spanish Speaker</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Maslak, Sarıyer/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>53 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Esvita Clinic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1316834</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316834</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Information Technology (IT) Analyst</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>124 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Özsayın Soğutma</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1296387</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1296387</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Şehitkamil, Türkiye</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>80 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Big Brands Dış Ticaret Limited Şirketi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-14 07:07:08 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -445,17 +445,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="71" customWidth="1" min="3" max="3"/>
-    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,64 +503,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1338354</t>
+          <t>1340218</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338354</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340218</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[DGF] Inside Sales Intern l German Speaker (EU Only)</t>
+          <t>[Impact Brazil] - Software Development Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mainz, Germany</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Chapecó, SC, Brasil</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>70 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DHL Group</t>
+          <t>BAUSER Construção Inteligente</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1338472</t>
+          <t>1340203</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338472</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340203</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[EXP] Intern - Customer Emission Reporting</t>
+          <t>Taste Hungary | Technical Customer Support Intern (EU ONLY)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>117 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -580,71 +580,71 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DHL Group</t>
+          <t>EATON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340175</t>
+          <t>1340202</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340175</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340202</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Accelerate Romania - Junior Marketing &amp; Growth Specialist</t>
+          <t>Taste Hungary | Customer Support Intern (EU preferred)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Baia Mare, Romania</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Coach Jurnal</t>
+          <t>EATON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340039</t>
+          <t>1340117</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340039</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340117</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Junior Hardware Engineer (EPLAN) – Marine Automation (Preferably EU)</t>
+          <t>Digital marketing</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Delft, Nederland</t>
+          <t>Ariana, Tunisie</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,39 +654,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Smart-Ship B.V.</t>
+          <t>Jardin d'enfants Meriem</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1338115</t>
+          <t>1338677</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338115</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338677</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[Remote] Software Application Support and Development</t>
+          <t>graphic designer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No location available</t>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -696,353 +696,59 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>126 applicants</t>
+          <t>7 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>dJava Factory Sdn Bhd</t>
+          <t>Eureka pharmaceuticals</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1336624</t>
+          <t>1334716</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336624</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334716</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Business Development Executive</t>
+          <t>[SNL] Global Talent Acquisition (EU citizen preferred)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Galle, Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>17 applicants</t>
+          <t>32 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Sanmark Solutions Pvt Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1336109</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336109</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Data Science Research Intern</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Sohna, Haryana 122103, India</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>10 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>K.R. Mangalam University</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1336107</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336107</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Cyber Security Research Intern</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Sohna, Haryana 122103, India</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>18 applicants</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>K.R. Mangalam University</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1336106</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336106</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence Research Intern</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Sohna, Haryana 122103, India</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>12 applicants</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>K.R. Mangalam University</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1327760</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1327760</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Fashion Consultant</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10 applicants</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>MPF clothing collection PVT LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1325297</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1325297</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>International Sales Representetive Spanish Speaker</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Maslak, Sarıyer/İstanbul, Türkiye</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>53 applicants</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Esvita Clinic</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1316834</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1316834</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Information Technology (IT) Analyst</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>124 applicants</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Özsayın Soğutma</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1296387</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1296387</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Şehitkamil, Türkiye</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>80 applicants</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Big Brands Dış Ticaret Limited Şirketi</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-15 06:49:28 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -79,7 +73,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340218</t>
+          <t>1340243</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340218</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340243</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[Impact Brazil] - Software Development Intern</t>
+          <t>Marketing Analyst Specialities and Oncology</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chapecó, SC, Brasil</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -533,44 +526,44 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BAUSER Construção Inteligente</t>
+          <t>GSK Panama</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340203</t>
+          <t>1338369</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340203</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338369</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Taste Hungary | Technical Customer Support Intern (EU ONLY)</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Coventry, UK</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>139 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -580,71 +573,71 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EATON</t>
+          <t>YBRANT CORE LIMITED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340202</t>
+          <t>1338279</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340202</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338279</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Taste Hungary | Customer Support Intern (EU preferred)</t>
+          <t>Client Services Executive</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Nugegoda, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EATON</t>
+          <t>Brand Corridor (Pvt) Ltd</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340117</t>
+          <t>1335628</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340117</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335628</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital marketing</t>
+          <t>Digital Marketer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ariana, Tunisie</t>
+          <t>Rades, Tunisia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>35 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -664,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Jardin d'enfants Meriem</t>
+          <t>AmazingPandph Digital Media Management</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1338677</t>
+          <t>1334000</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338677</t>
+          <t>https://aiesec.org/opportunity/global-talent/1334000</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>graphic designer</t>
+          <t>Social Media Marketing</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
+          <t>Piraeus, Greece</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -696,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7 applicants</t>
+          <t>92 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -706,49 +699,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Eureka pharmaceuticals</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1334716</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334716</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>[SNL] Global Talent Acquisition (EU citizen preferred)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>32 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>DHL Group</t>
+          <t>Supreme Yachting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-16 06:45:28 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="49" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340243</t>
+          <t>1340278</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340243</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340278</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Marketing Analyst Specialities and Oncology</t>
+          <t>Institute Engagement &amp; Partnerships Associate</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Mumbai, Maharashtra, India</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>GSK Panama</t>
+          <t>FUTURE VARSITY EDUCON LLP</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1338369</t>
+          <t>1340271</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338369</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340271</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Account Management Business Process Analyst</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Coventry, UK</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>139 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>YBRANT CORE LIMITED</t>
+          <t>G4S Panamá</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1338279</t>
+          <t>1340247</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338279</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340247</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Client Services Executive</t>
+          <t>Front Office Executive</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>New Delhi, Delhi, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Brand Corridor (Pvt) Ltd</t>
+          <t>Indian Hotels Company Private Limited</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1335628</t>
+          <t>1340246</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335628</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340246</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Marketer</t>
+          <t>Stewardess / Hostess - Food &amp; Beverage Service</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rades, Tunisia</t>
+          <t>New Delhi, Delhi, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>35 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>AmazingPandph Digital Media Management</t>
+          <t>Indian Hotels Company Private Limited</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1334000</t>
+          <t>1340245</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334000</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340245</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Social Media Marketing</t>
+          <t>Marketing Analyst</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Piraeus, Greece</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,17 +689,311 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>92 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sanfer Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1340173</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340173</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Financial analysis intern</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ambala, Haryana, India</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Supreme Yachting</t>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MM(DU) Mullana</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1339462</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339462</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>App Developer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Cairo, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>18 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Candy Clan Studios</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1339452</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339452</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Human Resource Research Intern - 6 Weeks</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1339180</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339180</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ankara, Türkiye</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>36 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>AHED Plastik</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1336043</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Digital Marketing &amp; Media Buying Specialist</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>17 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NOYO For Cosmetics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1331015</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331015</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sincan, İstasyon, 06934 Sincan/Ankara, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>103 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Maksan Lift</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1329104</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1329104</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sales Intern</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Pannipitiya, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>60 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Frella International</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-17 06:31:56 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
+    <col width="61" customWidth="1" min="3" max="3"/>
+    <col width="79" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340278</t>
+          <t>1340290</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340278</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340290</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Institute Engagement &amp; Partnerships Associate</t>
+          <t>AI-powered software development</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra, India</t>
+          <t>Tunis, Tunisia</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,34 +526,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FUTURE VARSITY EDUCON LLP</t>
+          <t>Legal Crea</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340271</t>
+          <t>1340286</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340271</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340286</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Account Management Business Process Analyst</t>
+          <t>Digital Marketer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Tunis, Tunisia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,34 +568,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>G4S Panamá</t>
+          <t>Legal Crea</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340247</t>
+          <t>1340210</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340247</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340210</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Front Office Executive</t>
+          <t>Accelerate Romania - Junior International Sales Specialist</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi, India</t>
+          <t>Cluj-Napoca, Romania</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Indian Hotels Company Private Limited</t>
+          <t>Cicada Technologies</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340246</t>
+          <t>1340207</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340246</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340207</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stewardess / Hostess - Food &amp; Beverage Service</t>
+          <t>Accelerate Romania - Junior QA &amp; Product Testing Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi, India</t>
+          <t>Cluj-Napoca, Romania</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Indian Hotels Company Private Limited</t>
+          <t>SiteCentric</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1340245</t>
+          <t>1340190</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340245</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340190</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing Analyst</t>
+          <t>Marketing Specialist</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Sanfer Panama</t>
+          <t>circle_realestate</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1340173</t>
+          <t>1339870</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340173</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339870</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Financial analysis intern</t>
+          <t>Project Specialist</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ambala, Haryana, India</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,39 +731,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>53 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MM(DU) Mullana</t>
+          <t>NESTRADE S.A, PANAMA BRANCH</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339462</t>
+          <t>1339262</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339462</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339262</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>App Developer</t>
+          <t>Mechanical Engineer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,39 +773,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>18 applicants</t>
+          <t>11 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Candy Clan Studios</t>
+          <t>Ray IC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1339452</t>
+          <t>1339260</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339452</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339260</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Human Resource Research Intern - 6 Weeks</t>
+          <t>Architecture Engineer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,39 +815,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>Ray IC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1339180</t>
+          <t>1339259</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339180</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339259</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Business Development</t>
+          <t>Electrical Engineer</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ankara, Türkiye</t>
+          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,39 +857,39 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>36 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>AHED Plastik</t>
+          <t>Ray IC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1336043</t>
+          <t>1337432</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337432</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Digital Marketing &amp; Media Buying Specialist</t>
+          <t>Junior Motion Graphic Designer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>6th of October City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,29 +909,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NOYO For Cosmetics</t>
+          <t>Olven White</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1331015</t>
+          <t>1337431</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331015</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337431</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Junior Motion Graphic Designer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sincan, İstasyon, 06934 Sincan/Ankara, Türkiye</t>
+          <t>6th of October City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,39 +941,39 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>103 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Maksan Lift</t>
+          <t>Olven White</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1329104</t>
+          <t>1337430</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329104</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337430</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sales Intern</t>
+          <t>Junior Account Manager</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pannipitiya, Sri Lanka</t>
+          <t>6th of October City, Giza Governorate, Egypt</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -983,17 +983,59 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>60 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Frella International</t>
+          <t>Olven White</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1334455</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334455</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Architecture Intern</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>M.A.H.E.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-18 06:59:54 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
-    <col width="79" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340290</t>
+          <t>1340189</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340290</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340189</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AI-powered software development</t>
+          <t>Marketing Specialist</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tunis, Tunisia</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Legal Crea</t>
+          <t>circle_realestate</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340286</t>
+          <t>1340161</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340286</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340161</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Digital Marketer</t>
+          <t>Operation Specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tunis, Tunisia</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Legal Crea</t>
+          <t>circle_realestate</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340210</t>
+          <t>1340159</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340210</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340159</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Accelerate Romania - Junior International Sales Specialist</t>
+          <t>Marketing &amp; Content Creation Specialist</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cluj-Napoca, Romania</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cicada Technologies</t>
+          <t>circle_realestate</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340207</t>
+          <t>1338821</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340207</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338821</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Accelerate Romania - Junior QA &amp; Product Testing Intern</t>
+          <t>Clinical Site Associate Trainee [ EU Only]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cluj-Napoca, Romania</t>
+          <t>1070 Anderlecht, Belgium</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>27 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SiteCentric</t>
+          <t>UCB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1340190</t>
+          <t>1337417</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340190</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337417</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing Specialist</t>
+          <t>AI Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>24 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>circle_realestate</t>
+          <t>E.C.O</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339870</t>
+          <t>1336115</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339870</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336115</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Project Specialist</t>
+          <t>Law Research Intern</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,311 +731,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>53 applicants</t>
+          <t>7 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NESTRADE S.A, PANAMA BRANCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1339262</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339262</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Mechanical Engineer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>11 applicants</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Ray IC</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1339260</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339260</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Architecture Engineer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Ray IC</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1339259</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339259</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Electrical Engineer</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Al Muqattam City, Al Abageyah, El Mokattam, Cairo Governorate 4414131, Egypt</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>4 applicants</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Ray IC</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1337432</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337432</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Junior Motion Graphic Designer</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Olven White</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1337431</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337431</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Junior Motion Graphic Designer</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Olven White</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1337430</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337430</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Junior Account Manager</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>6th of October City, Giza Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>3 applicants</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Olven White</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1334455</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334455</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Architecture Intern</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Manipal, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0 applicants</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>M.A.H.E.</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-19 07:11:14 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340189</t>
+          <t>1340123</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340189</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340123</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Marketing Specialist</t>
+          <t>Digital Marketing Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Kalpitiya, Sri Lanka</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>circle_realestate</t>
+          <t>Kitesurfing Lanka (Pvt) Limited</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340161</t>
+          <t>1337761</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340161</t>
+          <t>https://aiesec.org/opportunity/global-talent/1337761</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Operation Specialist</t>
+          <t>Export Manager Assistant</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>İzmir, Türkiye</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>132 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>circle_realestate</t>
+          <t>ACUNAL GIDA TARIM ÜRÜNLERİ MAKİNA İTHALAT İHRACAT SANAYİ VE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340159</t>
+          <t>1331631</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340159</t>
+          <t>https://aiesec.org/opportunity/global-talent/1331631</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Marketing &amp; Content Creation Specialist</t>
+          <t>developer mobile</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Sfax, Tunisie</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>36 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>circle_realestate</t>
+          <t>Sky Academy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338821</t>
+          <t>1329565</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338821</t>
+          <t>https://aiesec.org/opportunity/global-talent/1329565</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Clinical Site Associate Trainee [ EU Only]</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1070 Anderlecht, Belgium</t>
+          <t>Sfax, Tunisia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,101 +647,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>27 applicants</t>
+          <t>17 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>UCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1337417</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337417</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>AI Intern</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>24 applicants</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>E.C.O</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1336115</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336115</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Law Research Intern</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Sohna, Haryana 122103, India</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>7 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>K.R. Mangalam University</t>
+          <t>SRTC Country tunisia city sfax</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-20 06:57:15 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="63" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340123</t>
+          <t>1340219</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340123</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340219</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Digital Marketing Intern</t>
+          <t>Industrial Engineering Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kalpitiya, Sri Lanka</t>
+          <t>Bizerte, Tunisia</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Kitesurfing Lanka (Pvt) Limited</t>
+          <t>societe Precimeca</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1337761</t>
+          <t>1340125</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337761</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340125</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Export Manager Assistant</t>
+          <t>Business Coordinator Intern- GSP Compass</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>İzmir, Türkiye</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>132 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ACUNAL GIDA TARIM ÜRÜNLERİ MAKİNA İTHALAT İHRACAT SANAYİ VE</t>
+          <t>Euroasia Minmet Corp.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1331631</t>
+          <t>1339613</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1331631</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339613</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>developer mobile</t>
+          <t>Product Coordinator Intern – Digital Platform</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sfax, Tunisie</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>36 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Sky Academy</t>
+          <t>Euroasia Minmet Corp.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1329565</t>
+          <t>1338602</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329565</t>
+          <t>https://aiesec.org/opportunity/global-talent/1338602</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>social media specialist</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sfax, Tunisia</t>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>17 applicants</t>
+          <t>8 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,7 +657,133 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SRTC Country tunisia city sfax</t>
+          <t>Techno Genius</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1337797</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337797</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sales Representitive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Istanbul, İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>125 applicants</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aksan Kozmetik</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1337613</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337613</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cyberjaya, Selangor, Malaysia</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>188 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>IX Telecom Sdn Bhd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1336922</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336922</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sales Representitve</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Istanbul, İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>93 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KARTEK PASLANMAZ DEMİR İNŞAAT TAAHHÜT SANAYİ VE TİCARET LİMİ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-21 06:57:47 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,13 +438,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340219</t>
+          <t>1340416</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340219</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340416</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Industrial Engineering Intern</t>
+          <t>W2 Regional audit assistant</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bizerte, Tunisia</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>societe Precimeca</t>
+          <t>HILTI Panama</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340125</t>
+          <t>1340409</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340125</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340409</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Business Coordinator Intern- GSP Compass</t>
+          <t>[IMPACT FORTALEZA] Human Resources and Recruitment</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Castanhal, Pará, Brazil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Euroasia Minmet Corp.</t>
+          <t>Petruz Fruity</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339613</t>
+          <t>1340406</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339613</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340406</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Product Coordinator Intern – Digital Platform</t>
+          <t>[IMPACT FORTALEZA] Sales Operations Analyst</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Castanhal, Pará, Brazil</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Euroasia Minmet Corp.</t>
+          <t>Petruz Fruity</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1338602</t>
+          <t>1340405</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338602</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340405</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>social media specialist</t>
+          <t>[IMPACT FORTALEZA] Chemical Engineering and Food Formulation Engineering</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
+          <t>Castanhal, Pará, Brazil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Techno Genius</t>
+          <t>Petruz Fruity</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1337797</t>
+          <t>1339601</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337797</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339601</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sales Representitive</t>
+          <t>Female Guest Relations Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Istanbul, İstanbul, Türkiye</t>
+          <t>Nugegoda, Sri Lanka</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>125 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Aksan Kozmetik</t>
+          <t>Lanka Island Resorts Ltd.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1337613</t>
+          <t>1339486</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337613</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339486</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marketing Intern</t>
+          <t>IT (6 weeks!)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cyberjaya, Selangor, Malaysia</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,39 +731,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>188 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>IX Telecom Sdn Bhd</t>
+          <t>home mart reality</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1336922</t>
+          <t>1339485</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336922</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339485</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sales Representitve</t>
+          <t>Sales (6 weeks!)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Istanbul, İstanbul, Türkiye</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,17 +773,227 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>93 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>home mart reality</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1339481</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339481</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Digital marketing  (6 weeks!)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>home mart reality</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1338136</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338136</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Digital Communication Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Santiago do Cacém, Portugal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>98 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Destilaria Black Pig Alentejo Unip. Lda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1337857</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337857</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Intern</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Charneca de Caparica, Portugal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>156 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Indústria dos Óculos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1336690</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336690</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Electrical Automation Responsible</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Başakşehir, Başak, 34490 Başakşehir/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>39 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>BİRES OTOMASYON VE MÜHENDİSLİK HİZMETLERİ SANAYİ TİCARET LİM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1329428</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1329428</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[IMPACT FORTALEZA] COST &amp; QUALITY PLANNING</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Castanhal, PA, Brasil</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>4 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>6 - 18 Months</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>KARTEK PASLANMAZ DEMİR İNŞAAT TAAHHÜT SANAYİ VE TİCARET LİMİ</t>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Petruz Fruity</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-22 07:00:57 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="75" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="63" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340416</t>
+          <t>1340399</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340416</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340399</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>W2 Regional audit assistant</t>
+          <t>Web Development Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Al Obour City, Obour, Al-Qalyubia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>HILTI Panama</t>
+          <t>Hajjo Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340409</t>
+          <t>1340397</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340409</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340397</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[IMPACT FORTALEZA] Human Resources and Recruitment</t>
+          <t>Marketing Coordinator</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Castanhal, Pará, Brazil</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Petruz Fruity</t>
+          <t>Crizac Limited</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340406</t>
+          <t>1340359</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340406</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340359</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[IMPACT FORTALEZA] Sales Operations Analyst</t>
+          <t>Business Development Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Castanhal, Pará, Brazil</t>
+          <t>Al Obour City, Obour, Al-Qalyubia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Petruz Fruity</t>
+          <t>Hajjo Group</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340405</t>
+          <t>1340265</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340405</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340265</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[IMPACT FORTALEZA] Chemical Engineering and Food Formulation Engineering</t>
+          <t>Illustrator / Copywriter Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Castanhal, Pará, Brazil</t>
+          <t>Chennai, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Petruz Fruity</t>
+          <t>Whoa Mama</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339601</t>
+          <t>1336109</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339601</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336109</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Female Guest Relations Intern</t>
+          <t>Data Science Research Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nugegoda, Sri Lanka</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>12 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Lanka Island Resorts Ltd.</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1339486</t>
+          <t>1335631</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339486</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335631</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>IT (6 weeks!)</t>
+          <t>content creator</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Tunis, Tunisie</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>24 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +741,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>home mart reality</t>
+          <t>citywork Business Center</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1339485</t>
+          <t>1335630</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339485</t>
+          <t>https://aiesec.org/opportunity/global-talent/1335630</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sales (6 weeks!)</t>
+          <t>community manager</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Tunis, Tunisie</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>10 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,217 +783,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>home mart reality</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1339481</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339481</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Digital marketing  (6 weeks!)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1 applicant</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>home mart reality</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1338136</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338136</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Digital Communication Intern</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Santiago do Cacém, Portugal</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>98 applicants</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Destilaria Black Pig Alentejo Unip. Lda.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1337857</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337857</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence Intern</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Charneca de Caparica, Portugal</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>156 applicants</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>9 - 12 Weeks</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Indústria dos Óculos</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1336690</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336690</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Electrical Automation Responsible</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Başakşehir, Başak, 34490 Başakşehir/İstanbul, Türkiye</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>39 applicants</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>BİRES OTOMASYON VE MÜHENDİSLİK HİZMETLERİ SANAYİ TİCARET LİM</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1329428</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1329428</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>[IMPACT FORTALEZA] COST &amp; QUALITY PLANNING</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Castanhal, PA, Brasil</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>4 applicants</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>6 - 18 Months</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Petruz Fruity</t>
+          <t>citywork Business Center</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-23 06:56:49 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340399</t>
+          <t>1340475</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340399</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340475</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Web Development Intern</t>
+          <t>Community Business Development &amp; Partnerships Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Al Obour City, Obour, Al-Qalyubia Governorate, Egypt</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Hajjo Group</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340397</t>
+          <t>1340473</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340397</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340473</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Marketing Coordinator</t>
+          <t>Social Research &amp; Innovation Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Crizac Limited</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340359</t>
+          <t>1340472</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340359</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340472</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Business Development Intern</t>
+          <t>Digital Content &amp; Social Media Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Al Obour City, Obour, Al-Qalyubia Governorate, Egypt</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Hajjo Group</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340265</t>
+          <t>1340471</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340265</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340471</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Illustrator / Copywriter Intern</t>
+          <t>International Community Engagement Intern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu, India</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -652,34 +652,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Whoa Mama</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1336109</t>
+          <t>1340470</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336109</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340470</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Data Science Research Intern</t>
+          <t>Biodiversity &amp; Environmental Education Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>12 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1335631</t>
+          <t>1340469</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335631</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340469</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>content creator</t>
+          <t>Environmental Education and Sustainability Intern</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tunis, Tunisie</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>24 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -741,29 +741,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>citywork Business Center</t>
+          <t>Onevaasa Wilderness Labs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1335630</t>
+          <t>1340460</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1335630</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340460</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>community manager</t>
+          <t>Sustainable Tourism &amp; Community Development Intern</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tunis, Tunisie</t>
+          <t>Ranchi, Jharkhand, India</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,7 +783,763 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>citywork Business Center</t>
+          <t>Onevaasa Wilderness Labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1340247</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340247</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Front Office Executive</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi, India</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Indian Hotels Company Private Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1338950</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338950</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[Impact Brazil] - E-Commerce Creative Content &amp; Listing Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Uberlândia, Minas Gerais, Brazil</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>30 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PAT E-Commerce &amp; International Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1338306</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338306</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>People Team Analyst</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>86 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1337537</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337537</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sales Responsible</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Konya, Türkiye</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>85 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TBPART OTOMOTİV SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1336121</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336121</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Economics Research Intern</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1336119</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336119</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Game Design Research Intern</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1336118</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336118</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Forensic Science Research Intern</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1336117</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336117</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UI/UX Research Intern</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1 applicant</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1336116</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336116</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hotel Management Research Intern</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1336114</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336114</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pharmacy Research Intern</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>4 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1336113</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336113</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>International Accounting Research Intern</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1336112</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336112</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Business Administration Research Intern</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1336111</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336111</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Computer Science Engineering Research Intern</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>5 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1336110</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336110</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Human Resource Research Intern</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1336108</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336108</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Full Stack Development Research Intern</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>7 applicants</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1336107</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336107</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cyber Security Research Intern</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>18 applicants</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1336104</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336104</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Finance Research Intern</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>14 applicants</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1296387</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1296387</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Şehitkamil, Türkiye</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>81 applicants</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Big Brands Dış Ticaret Limited Şirketi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-25 07:11:06 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -443,12 +443,12 @@
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="51" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340428</t>
+          <t>1340446</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340428</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340446</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Strategic Marketer</t>
+          <t>App Developer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tunis, Tunisia</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>La fabrique</t>
+          <t>Candy Clan Studios</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340388</t>
+          <t>1340380</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340388</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340380</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mechanical Engineering  Intern</t>
+          <t>Marketing specialist</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bizerte</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,34 +568,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>societe Precimeca</t>
+          <t>MS Technologies</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340055</t>
+          <t>1339060</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340055</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339060</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>interior architect</t>
+          <t>Graphic designer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sousse, Tunisie</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Zitouni Interior</t>
+          <t>Clicks Creative Agency</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339446</t>
+          <t>1336047</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339446</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336047</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Full Stack Development Research Intern - 6 Weeks</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>21 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>NOYO For Cosmetics</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339433</t>
+          <t>1336045</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339433</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336045</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Data Science Research Intern - 6 Weeks</t>
+          <t>Motion Graphics Designer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,39 +689,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>NOYO For Cosmetics</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1310446</t>
+          <t>1336043</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1310446</t>
+          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Education Coordinator</t>
+          <t>Digital Marketing &amp; Media Buying Specialist</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bursa, Türkiye</t>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>46 applicants</t>
+          <t>17 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Genç Kardelen Kindergarden</t>
+          <t>NOYO For Cosmetics</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-26 07:21:04 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,17 +496,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340446</t>
+          <t>1340467</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340446</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340467</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>App Developer</t>
+          <t>Automation engineer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,24 +531,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Candy Clan Studios</t>
+          <t>SETRA for Contracting &amp; Trading</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340380</t>
+          <t>1340464</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340380</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340464</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Marketing specialist</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>MS Technologies</t>
+          <t>Origin by Sherif</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339060</t>
+          <t>1339871</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339060</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339871</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Graphic designer</t>
+          <t>Application Security (AppSec) Engineer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Cairo, Cairo Governorate, Egypt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>9 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Clicks Creative Agency</t>
+          <t>Riva Talent</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1336047</t>
+          <t>1339451</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336047</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339451</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>Hotel Management Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>21 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NOYO For Cosmetics</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1336045</t>
+          <t>1339340</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336045</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339340</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Motion Graphics Designer</t>
+          <t>Artificial Intelligence Research Intern 6 weeks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,59 +689,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NOYO For Cosmetics</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1336043</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Digital Marketing &amp; Media Buying Specialist</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>New Cairo City, Cairo Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>17 applicants</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>3 - 6 Months</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>NOYO For Cosmetics</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-27 07:13:57 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="71" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="43" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340467</t>
+          <t>1340557</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340467</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340557</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation engineer</t>
+          <t>Guest Relations</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Phu Quoc, An Giang, Vietnam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -531,29 +531,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SETRA for Contracting &amp; Trading</t>
+          <t>Crowne Plaza</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340464</t>
+          <t>1340556</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340464</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340556</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Food &amp; Beverage</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Phu Quoc, An Giang, Vietnam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -573,29 +573,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Origin by Sherif</t>
+          <t>Crowne Plaza</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1339871</t>
+          <t>1340555</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339871</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340555</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Application Security (AppSec) Engineer</t>
+          <t>Recreation</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Phu Quoc, An Giang, Vietnam</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>9 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Riva Talent</t>
+          <t>Crowne Plaza</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1339451</t>
+          <t>1340552</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339451</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340552</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hotel Management Research Intern - 6 Weeks</t>
+          <t>Order-to-Invoice Trainee [EU Only]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>Sofia, Bulgaria</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>dormakaba</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1339340</t>
+          <t>1340530</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1339340</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340530</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Artificial Intelligence Research Intern 6 weeks</t>
+          <t>Accelerate Romania - Junior Social Media Content Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sohna, Haryana 122103, India</t>
+          <t>Cluj-Napoca, Romania</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,7 +699,259 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>K.R. Mangalam University</t>
+          <t>Antidot</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1340416</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340416</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>W2 Regional audit assistant</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>HILTI Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1340267</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340267</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sales Marketeer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rotterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>11 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>USP Marketing Consultancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1340039</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340039</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Junior Hardware Engineer (EPLAN) – Marine Automation (Preferably EU)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Delft, Nederland</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>56 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Smart-Ship B.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1338121</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338121</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Marketing/Graphic Design Intern</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Santiago do Cacém, Portugal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>39 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Destilaria Black Pig Alentejo Unip. Lda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1336200</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336200</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Business Development Executive (Remote)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Islamabad, Pakistan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>35 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Dunya Consultants</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1334523</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1334523</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Biotechnology Intern</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Manipal, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>7 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>MAHE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-28 07:47:41 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="71" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="43" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340557</t>
+          <t>1340606</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340557</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340606</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Guest Relations</t>
+          <t>[Impact Brazil] - Project Management Intern</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Phu Quoc, An Giang, Vietnam</t>
+          <t>Joinville - Pirabeiraba, Joinville - Santa Catarina, Brazil</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Crowne Plaza</t>
+          <t>Nidec Global Appliance</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340556</t>
+          <t>1340545</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340556</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340545</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Food &amp; Beverage</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Phu Quoc, An Giang, Vietnam</t>
+          <t>Pančevo, Serbia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>12 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Crowne Plaza</t>
+          <t>NETWORK MANAGER DOO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340555</t>
+          <t>1340521</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340555</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340521</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Recreation</t>
+          <t>Marketing and Strategy Intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Phu Quoc, An Giang, Vietnam</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -610,34 +610,34 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>3 - 6 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Crowne Plaza</t>
+          <t>Credifin Limited</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340552</t>
+          <t>1339456</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340552</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339456</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Order-to-Invoice Trainee [EU Only]</t>
+          <t>UI/UX Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sofia, Bulgaria</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,39 +647,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>5 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>dormakaba</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1340530</t>
+          <t>1339455</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340530</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339455</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Accelerate Romania - Junior Social Media Content Intern</t>
+          <t>Pharmacy Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cluj-Napoca, Romania</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>5 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -699,29 +699,29 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Antidot</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1340416</t>
+          <t>1339454</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340416</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339454</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>W2 Regional audit assistant</t>
+          <t>Law Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -736,34 +736,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>HILTI Panama</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1340267</t>
+          <t>1339453</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340267</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339453</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sales Marketeer</t>
+          <t>International Accounting Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Rotterdam, Netherlands</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -773,39 +773,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>USP Marketing Consultancy</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1340039</t>
+          <t>1339452</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340039</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339452</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Junior Hardware Engineer (EPLAN) – Marine Automation (Preferably EU)</t>
+          <t>Human Resource Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Delft, Nederland</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -815,39 +815,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>56 applicants</t>
+          <t>11 applicants</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Smart-Ship B.V.</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1338121</t>
+          <t>1339442</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338121</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339442</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Marketing/Graphic Design Intern</t>
+          <t>Forensic Science Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Santiago do Cacém, Portugal</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>39 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Destilaria Black Pig Alentejo Unip. Lda.</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1336200</t>
+          <t>1339441</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1336200</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339441</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Business Development Executive (Remote)</t>
+          <t>Finance Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>35 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,29 +909,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Dunya Consultants</t>
+          <t>K.R. Mangalam University</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1334523</t>
+          <t>1339435</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1334523</t>
+          <t>https://aiesec.org/opportunity/global-talent/1339435</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Biotechnology Intern</t>
+          <t>Economics Research Intern - 6 Weeks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Manipal, Karnataka, India</t>
+          <t>Sohna, Haryana 122103, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -941,17 +941,395 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>7 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1339392</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339392</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Business Administration Research Intern - 6 Weeks</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1339083</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1339083</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cyber Security Research Intern - 6 Weeks</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sohna, Haryana 122103, India</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>13 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>K.R. Mangalam University</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1338045</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338045</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Accelerate Romania | Back-end Developer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Timișoara, România</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>99 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Webchain</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1337434</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337434</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Customer Success Executive</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Córdoba, Argentina</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>94 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Teleprom Argentina S.A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1337411</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1337411</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Guest Experience Manager</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nugegoda, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>24 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>3 - 6 Months</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>MAHE</t>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Indian Kitchen (Pvt) Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1332481</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332481</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Market Researcher</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>161 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ÖZÇELİK MAKİNA SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1332359</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1332359</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sales Manager at Bİ-PLAST PLASTİK</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Adana, Reşatbey, Seyhan/Adana, Türkiye</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>28 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bİ-PLAST-PLASTİK</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1324350</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1324350</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Inbound Tour Executive - Mid Term</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Nugegoda, Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>12 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Trotter Escapes (Pvt) Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1316099</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316099</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sales &amp; BD Junior Manager</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Puzi City, Chiayi County, Taiwan 613</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>137 applicants</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Singform Enterprise Co., Ltd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-30 08:11:59 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -438,17 +438,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="152" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,22 +496,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340631</t>
+          <t>1340664</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340631</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340664</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Accelerate Romania |Sales Specialist Intern</t>
+          <t>Jr Customer Service Assistant</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Oradea, România</t>
+          <t>Leon, Guanajuato, Mexico</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,39 +521,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3 applicants</t>
+          <t>4 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>QuartzDevs SRL</t>
+          <t>CZR Consulting S.C.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340628</t>
+          <t>1340663</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340628</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340663</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Accelerate Romania | Marketing &amp; Content Intern</t>
+          <t>Sr Logistic Associate</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Oradea, România</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,39 +563,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>8 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>QuartzDevs SRL</t>
+          <t>Samsung Electronics Latinoamerica SELA Panama</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340079</t>
+          <t>1340662</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340079</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340662</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Digital Marketer</t>
+          <t>MIS - IT Sr Support</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cairo, Cairo Governorate, Egypt</t>
+          <t>Panamá, Provincia de Panamá, Panamá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,39 +605,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0 applicants</t>
+          <t>1 applicant</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Utopia advertising Egypt</t>
+          <t>Samsung Electronics Latinoamerica SELA Panama</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1337808</t>
+          <t>1340618</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1337808</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340618</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sales &amp; Impact Trainee</t>
+          <t>Associate, Client Service, 2027 [Hiring for Japanese / Vietnamese / Thai / Mandarin / Korean / Tagalog / Bahasa Indonesia / English / Hindi speakers]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>135 applicants</t>
+          <t>6 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +657,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Shayp</t>
+          <t>AlphaSights</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1321076</t>
+          <t>1340554</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1321076</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340554</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Corporate Sales Executive</t>
+          <t>Social Media Specialist / Strategist</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mehrauli, Delhi, India</t>
+          <t>Tanta, Tanta Qism 2, Tanta, Gharbia Governorate, Egypt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -689,17 +689,101 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6 - 18 Months</t>
+          <t>9 - 12 Weeks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Empathy Relocations</t>
+          <t>Pavone medical center</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1338950</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338950</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[Impact Brazil] - E-Commerce Creative Content &amp; Listing Marketing Intern</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Uberlândia, Minas Gerais, Brazil</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>32 applicants</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PAT E-Commerce &amp; International Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1338676</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338676</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data analysist</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>53 applicants</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Eureka pharmaceuticals</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel files after daily scrape - 2026-10-31 07:59:12 UTC
</commit_message>
<xml_diff>
--- a/New.xlsx
+++ b/New.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +79,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,17 +445,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="152" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="59" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,32 +503,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1340664</t>
+          <t>1340737</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340664</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340737</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jr Customer Service Assistant</t>
+          <t>[SNL] Intern Digital HR Communications &amp; User Experience</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Leon, Guanajuato, Mexico</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Charles-de-Gaulle-Straße 20, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 applicants</t>
+          <t>3 applicants</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,39 +538,39 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CZR Consulting S.C.</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1340663</t>
+          <t>1340734</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340663</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340734</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sr Logistic Associate</t>
+          <t>[EXP NL] Data Science Intern</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Maastricht, Netherlands</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 applicants</t>
+          <t>7 applicants</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -573,29 +580,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+          <t>DHL Group</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1340662</t>
+          <t>1340718</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340662</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340718</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MIS - IT Sr Support</t>
+          <t>Learning and development intern</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Panamá, Provincia de Panamá, Panamá</t>
+          <t>Panama City, Panamá Province, Panama</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -605,7 +612,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 applicant</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,29 +622,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Samsung Electronics Latinoamerica SELA Panama</t>
+          <t>HILTI Panama</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1340618</t>
+          <t>1340714</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340618</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340714</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Associate, Client Service, 2027 [Hiring for Japanese / Vietnamese / Thai / Mandarin / Korean / Tagalog / Bahasa Indonesia / English / Hindi speakers]</t>
+          <t>Technical Support Analyst-Perú</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Ciudad de Córdoba, Provincia de Córdoba, Argentina</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -647,7 +654,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6 applicants</t>
+          <t>0 applicants</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -657,29 +664,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>AlphaSights</t>
+          <t>Teleprom Argentina S.A</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1340554</t>
+          <t>1340713</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1340554</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340713</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Social Media Specialist / Strategist</t>
+          <t>AIESEC Junior Brand Manager Trainee [ EU Only ]</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tanta, Tanta Qism 2, Tanta, Gharbia Governorate, Egypt</t>
+          <t>1070 Anderlecht, Belgium</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -694,34 +701,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9 - 12 Weeks</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Pavone medical center</t>
+          <t>UCB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1338950</t>
+          <t>1340712</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338950</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340712</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[Impact Brazil] - E-Commerce Creative Content &amp; Listing Marketing Intern</t>
+          <t>Administration Analyst Perú</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Uberlândia, Minas Gerais, Brazil</t>
+          <t>Ciudad de Córdoba, Provincia de Córdoba, Argentina</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -731,59 +738,563 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>32 applicants</t>
+          <t>2 applicants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3 - 6 Months</t>
+          <t>6 - 18 Months</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PAT E-Commerce &amp; International Trade</t>
+          <t>Teleprom Argentina S.A</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1338676</t>
+          <t>1340700</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://aiesec.org/opportunity/global-talent/1338676</t>
+          <t>https://aiesec.org/opportunity/global-talent/1340700</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Data analysist</t>
+          <t>[DSC] Commercial Digital Transformation Intern</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mansoura, Mansoura Qism 2, El Mansoura, Dakahlia Governorate, Egypt</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Fritz-Erler-Straße 5, 53113 Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>53 applicants</t>
+          <t>10 applicants</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DHL Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1340528</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340528</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Telesales</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>9 - 12 Weeks</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Eureka pharmaceuticals</t>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EA2 Communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1340527</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340527</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EA2 Communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1340524</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1340524</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Account Executive</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Giza, El Omraniya, Giza Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0 applicants</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EA2 Communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1338585</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338585</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Furniture designer / Interior Designer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cairo, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6 applicants</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9 - 12 Weeks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>kremastos</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1338571</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1338571</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Product Catalog and Online Store</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>31073 Delligsen, Deutschland</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>140 applicants</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Bornemann Gewindetechnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1336045</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336045</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Motion Graphics Designer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>6 applicants</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NOYO For Cosmetics</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1336043</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1336043</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Digital Marketing &amp; Media Buying Specialist</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>New Cairo City, Cairo Governorate, Egypt</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>17 applicants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NOYO For Cosmetics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1331894</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331894</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sales Engineer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Kartepe, Kocaeli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>104 applicants</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3 - 6 Months</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Atom Mek</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1331267</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1331267</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sales Representative</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Dilovası, Kocaeli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>74 applicants</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>IPOS Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1322764</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1322764</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sales Engineering</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Çayırova, Kocaeli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>31 applicants</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ÇEL-MER ÇELİK ENDÜSTRİSİ ANONİM ŞİRKETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1316551</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1316551</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>İzmit, Kocaeli, Türkiye</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>111 applicants</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Akademi Hastanesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1296457</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://aiesec.org/opportunity/global-talent/1296457</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sales Engineering</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Dilovası, Türkiye</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>213 applicants</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>6 - 18 Months</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Eurotray Metal Elektrik Company</t>
         </is>
       </c>
     </row>

</xml_diff>